<commit_message>
Schema v2: add 7 new columns and backfill EOW-001 to EOW-015
New columns added to Escape_of_Water_Case_Database.xlsx:
  - Insurer Name
  - FOS Decision Date (accept-or-reject deadline from decision)
  - Dispute Type (Coverage / Handling / Endorsement / Pre-Inception /
                  Peril Classification / Admin / Broker Conduct)
  - Coverage Decision (Declined Full / Accepted / Disputed Settlement /
                       Not Applicable)
  - Outcome Category (Upheld / Upheld in Part / Not Upheld /
                      Compensation Only)
  - Compensation Awarded (£)
  - Is Core Case (Yes / No — with reason tag)

All 15 existing rows backfilled. Non-core flags applied:
  EOW-004 (Administrative), EOW-009 (Handling),
  EOW-014 (Commercial), EOW-015 (Broker Dispute).

Migration script: scripts/migrate_schema_v2.py

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/knowledge/case-databases/Escape_of_Water_Case_Database.xlsx
+++ b/knowledge/case-databases/Escape_of_Water_Case_Database.xlsx
@@ -470,23 +470,30 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:U16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
-    <col width="55" customWidth="1" min="7" max="7"/>
-    <col width="55" customWidth="1" min="8" max="8"/>
-    <col width="55" customWidth="1" min="9" max="9"/>
-    <col width="45" customWidth="1" min="10" max="10"/>
-    <col width="70" customWidth="1" min="11" max="11"/>
-    <col width="70" customWidth="1" min="12" max="12"/>
-    <col width="70" customWidth="1" min="13" max="13"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="25" customWidth="1" min="9" max="9"/>
+    <col width="50" customWidth="1" min="10" max="10"/>
+    <col width="55" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="55" customWidth="1" min="13" max="13"/>
     <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="55" customWidth="1" min="16" max="16"/>
+    <col width="45" customWidth="1" min="17" max="17"/>
+    <col width="70" customWidth="1" min="18" max="18"/>
+    <col width="70" customWidth="1" min="19" max="19"/>
+    <col width="70" customWidth="1" min="20" max="20"/>
+    <col width="22" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -502,60 +509,95 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Insurer Name</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>FOS Decision Date</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Claim Type</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Leak Source</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Property Type</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Dispute Type</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Coverage Decision</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Rejection Reason</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Evidence Dispute</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Outcome Category</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Outcome</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Compensation Awarded (£)</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Is Core Case</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Key Policy Clause</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Missing Evidence</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Ombudsman Reasoning</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Workflow Insight</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>AI Rule Candidate</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Source PDF</t>
         </is>
@@ -572,62 +614,95 @@
           <t>DRN-2088302</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Fairmead Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>11 Sep 2020</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>Escape of water — corroded underfloor pipe, floor and carpet damage</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>Corroded underground pipe beneath concrete living room floor (corrosion from concrete onto pipe)</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Residential home</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
         <is>
           <t>Initial full decline — insurer attributed damage to rising damp caused by absence of damp-proof membrane, not to escape of water from the pipe</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="K2" s="3" t="inlineStr">
         <is>
           <t>Customer provided photos of lifting laminate and displaced tiles in hallway. Insurer limited covered area to approx. 1/10 of total flooring replaced. Builder could not provide itemised breakdown separating covered works from DPM installation.</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Upheld in Part</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
         <is>
           <t>Upheld in part — insurer must settle claim for area directly damaged by escape of water (£260 concrete floor + £390 carpet less £600 excess = £50 net payment) plus £150 compensation for incorrectly declining in full</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="N2" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P2" s="3" t="inlineStr">
         <is>
           <t>Policy covers damage caused by escape of water but not rising damp. Trace and access not covered under this policy. Policy excess £600.</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr">
+      <c r="Q2" s="3" t="inlineStr">
         <is>
           <t>Itemised breakdown of builder's repair costs separating escape of water damage from DPM installation and general improvement works. Builder unable to provide further clarification.</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="R2" s="3" t="inlineStr">
         <is>
           <t>Escape of water was an insured event — not in dispute. Wider damage more likely caused by rising damp and absence of DPM. DPM installation is not a covered repair. Area directly damaged by escape of water limited to proximity of burst pipe. Laminate flooring replacement not proven necessary (waterproof underlay in place). Insurer's initial full decline was incorrect and caused distress warranting compensation.</t>
         </is>
       </c>
-      <c r="L2" s="3" t="inlineStr">
+      <c r="S2" s="3" t="inlineStr">
         <is>
           <t>Distinguish damage caused by escape of water from damage caused by rising damp or absence of maintenance features (e.g. DPM). Insurer must not decline in full if any part of damage is from an insured peril. Settlement quantum requires itemised separation of covered vs non-covered repair costs. Proximity of damage to pipe source is the key spatial evidence.</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
+      <c r="T2" s="3" t="inlineStr">
         <is>
           <t>If insurer declines in full but escape of water is confirmed, flag as improper full decline. Require itemised contractor breakdown separating escape of water damage from maintenance or improvement works. Apply coverage to area proximate to pipe source only.</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="U2" s="2" t="inlineStr">
         <is>
           <t>DRN-2088302.pdf</t>
         </is>
@@ -644,62 +719,95 @@
           <t>DRN-3258984</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>U K Insurance Limited (UKI)</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>30 Mar 2022</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
         <is>
           <t>Escape of water — post-repair deterioration and disputed scope of water damage</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="F3" s="5" t="inlineStr">
         <is>
           <t>Escape of water (December 2020) — original source accepted by insurer; subsequent dispute over whether additional floor areas were affected</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="G3" s="4" t="inlineStr">
         <is>
           <t>Residential home</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>Handling / Reinstatement Dispute</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>Accepted — Disputed Settlement</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
         <is>
           <t>Insurer declined to extend claim to front bedroom and landing floors — three separate independent contractor assessments found no water staining or swelling; insurer concluded floor movement was age-related wear and tear</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="K3" s="5" t="inlineStr">
         <is>
           <t>Customer's own report failed to establish causation for front bedroom/landing but confirmed ongoing floor movement in en suite and middle bedroom (areas originally repaired by insurer). Insurer argued customer's report did not attribute damage to the insured peril. No contractor lifted carpets during any of the three inspections.</t>
         </is>
       </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="L3" s="4" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M3" s="5" t="inlineStr">
         <is>
           <t>Upheld — UKI must reimburse cost of customer's independent report, carry out or pay for repairs to en suite and middle bedroom, pay £400 compensation (distress from incomplete original repair and unnecessary furniture removal instruction)</t>
         </is>
       </c>
-      <c r="I3" s="5" t="inlineStr">
+      <c r="N3" s="4" t="n">
+        <v>400</v>
+      </c>
+      <c r="O3" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P3" s="5" t="inlineStr">
         <is>
           <t>Coverage limited to areas demonstrably damaged by escape of water. Wear and tear excluded. Insurer obligated to carry out a full and lasting reinstatement.</t>
         </is>
       </c>
-      <c r="J3" s="5" t="inlineStr">
+      <c r="Q3" s="5" t="inlineStr">
         <is>
           <t>Carpets were not lifted during any of the three contractor inspections. No independent assessment of whether the original reinstatement was full and lasting before the complaint arose.</t>
         </is>
       </c>
-      <c r="K3" s="5" t="inlineStr">
+      <c r="R3" s="5" t="inlineStr">
         <is>
           <t>Three independent specialists found no evidence of water damage to front bedroom or landing — FOS accepted this area is not covered. Customer's own report confirmed post-repair movement in en suite and middle bedroom (originally repaired areas), indicating original repair was not full and lasting — these repairs remain claim-related. Insurer responsible for completing a proper reinstatement. Contractor telling customer to move furniture unnecessarily created additional distress liability. Vulnerable customer status relevant to compensation level.</t>
         </is>
       </c>
-      <c r="L3" s="5" t="inlineStr">
+      <c r="S3" s="5" t="inlineStr">
         <is>
           <t>Insurer must ensure reinstatement is full and lasting — subsequent deterioration in originally repaired areas remains claim-related. Multiple independent experts finding no water damage to specific areas is near-decisive evidence those areas are not covered. Contractor instructions to customers (e.g. clear a room) can create compensation liability if later unnecessary. Vulnerable customer status is a factor in assessing appropriate compensation.</t>
         </is>
       </c>
-      <c r="M3" s="5" t="inlineStr">
+      <c r="T3" s="5" t="inlineStr">
         <is>
           <t>If post-repair deterioration is reported in originally repaired areas, flag as potential incomplete reinstatement (still claim-related). Where three or more independent experts agree no water damage to a specific area, treat as near-decisive evidence against coverage of that area. Document all contractor instructions to customers — unnecessary actions generate distress liability.</t>
         </is>
       </c>
-      <c r="N3" s="4" t="inlineStr">
+      <c r="U3" s="4" t="inlineStr">
         <is>
           <t>DRN-3258984.pdf</t>
         </is>
@@ -716,62 +824,95 @@
           <t>DRN-4132443</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>QIC Europe Ltd</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>08 Jan 2024</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Escape of water — deteriorated underground drainage pipe, kitchen building and contents damage</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Cracked and deteriorated underground drainage pipe beneath kitchen floor</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Residential home (kitchen)</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>Full decline — insurer's drainage contractor (desk review only, no physical inspection) found no evidence of accidental damage. Insurer said pipe damage did not meet policy accidental damage definition and surveyor found no water damage in kitchen.</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>Builder's report confirmed kitchen water damage: floor grout darkened with mould, musty smell, base units and floor trims unfit for use. Customer provided video showing soaking wet flooring and photos of water damage. Insurer's surveyor noted damaged base units, worktop and floor tiles but did not opine on coverage. Insurer's drainage contractor conducted desk review of builder's report without physical inspection.</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
         <is>
           <t>Upheld — pipe repair fairly declined (gradual deterioration does not meet accidental damage definition). Escape of water damage to kitchen building and contents covered. Trace and access costs covered up to £10,000 policy limit (independent of pipe coverage). £200 compensation for distress and inconvenience.</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="N4" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P4" s="3" t="inlineStr">
         <is>
           <t>Accidental damage defined as: sudden, unexpected, physical damage at a specific time, not deliberate, caused by something external and identifiable. Trace and access covered up to £10,000 — triggered by existence of escape of water, not dependent on pipe claim succeeding.</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="Q4" s="3" t="inlineStr">
         <is>
           <t>Itemised breakdown of trace and access costs separate from pipe repair costs. Full assessment of remaining escape of water building and contents damage costs.</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="R4" s="3" t="inlineStr">
         <is>
           <t>Pipe was cracked and fallen apart with no specific cause identified — consistent with gradual deterioration, not accidental damage per policy definition. Escape of water from the pipe clearly caused kitchen building and contents damage — this is covered regardless of whether the pipe itself is covered. Trace and access is a standalone policy benefit triggered by the existence of an escape of water. Each coverage element (pipe, building, trace and access, contents) must be assessed independently. Insurer's reliance on desk review without physical inspection was insufficient to deny kitchen damage.</t>
         </is>
       </c>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="S4" s="3" t="inlineStr">
         <is>
           <t>Always assess each coverage element separately: (1) pipe/source damage, (2) escape of water building damage, (3) trace and access, (4) contents. Trace and access is a standalone benefit — it is triggered by escape of water existing, not by the pipe claim succeeding. Gradual deterioration of underground pipes typically fails the accidental damage definition. Builder's report confirming water damage should be accepted unless specifically contradicted by an independent physical inspection.</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
+      <c r="T4" s="3" t="inlineStr">
         <is>
           <t>Separate coverage assessment required for each element: pipe damage, building damage, trace and access, contents. Check whether trace and access is a standalone benefit in the policy. If underground pipe described as gradually deteriorated/cracked — likely decline on pipe, but assess escape of water damage and trace and access independently. Desk-review-only denial of escape of water building damage insufficient without physical inspection.</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr">
+      <c r="U4" s="2" t="inlineStr">
         <is>
           <t>DRN-4132443.pdf</t>
         </is>
@@ -788,62 +929,95 @@
           <t>DRN4969124</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>UK Insurance Limited (UKI)</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>27 Feb 2015</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>Escape of water — claim recording dispute (same incident recorded as two separate claims)</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>Water pipe embedded in kitchen wall (initially misidentified by customer as washing machine leak)</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>Residential home (kitchen)</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>Claim Recording / Administrative Dispute</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
         <is>
           <t>Not a coverage rejection — insurer recorded the same incident as two separate claims because it received two reports. This caused downstream policy voidance by a subsequent insurer and higher insurance premiums.</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="K5" s="5" t="inlineStr">
         <is>
           <t>Kitchen plan and photographs demonstrated how the misidentification of source was plausible. Insurer's own 2007 investigation report stated 'claim can be dealt with as one with one excess.' Insurer failed to act on its own assessment when recording the claims.</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M5" s="5" t="inlineStr">
         <is>
           <t>Upheld — UKI must amend all records to show a single claim for the 2007 escape of water. Must contact current insurer to request policy voidance record is removed. Must refund any additional costs or premiums incurred as a result of the two-claim recording.</t>
         </is>
       </c>
-      <c r="I5" s="5" t="inlineStr">
+      <c r="N5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" s="4" t="inlineStr">
+        <is>
+          <t>No — Administrative</t>
+        </is>
+      </c>
+      <c r="P5" s="5" t="inlineStr">
         <is>
           <t>Single incident principle — one source, one claim, one excess. Insurer's own investigation report acknowledged the incident should be treated as a single claim.</t>
         </is>
       </c>
-      <c r="J5" s="5" t="inlineStr">
+      <c r="Q5" s="5" t="inlineStr">
         <is>
           <t>Documented evidence of additional premium costs or financial losses directly caused by the two-claim recording.</t>
         </is>
       </c>
-      <c r="K5" s="5" t="inlineStr">
+      <c r="R5" s="5" t="inlineStr">
         <is>
           <t>Two reports arose from customer's misdiagnosis of the same underlying source. Failure of initial drying revealed the correct source — a pipe in the wall. Both reports related to the same escape of water incident. Insurer's own records explicitly acknowledged the incident could be treated as a single claim with one excess. Insurer was bound by its own assessment. Downstream consequences (policy voidance, higher premiums) flowed directly from the incorrect recording and are the insurer's responsibility to remedy.</t>
         </is>
       </c>
-      <c r="L5" s="5" t="inlineStr">
+      <c r="S5" s="5" t="inlineStr">
         <is>
           <t>Where two reports are received for the same property within a short period, assess whether they relate to the same underlying source and incident. Insurer's own investigation records that suggest a single incident are binding on the insurer. Incorrect multiple-claim recording can have serious downstream consequences (policy voidance, premium increases) that the insurer must actively remedy. Initial customer misdiagnosis of leak source does not create two separate claims.</t>
         </is>
       </c>
-      <c r="M5" s="5" t="inlineStr">
+      <c r="T5" s="5" t="inlineStr">
         <is>
           <t>If two claim reports received for same property within a short period, assess whether they relate to the same source/incident. Check insurer's investigation notes — if they indicate single incident, record as one claim. Flag if incorrect multiple-claim recording may adversely affect customer's claims history or future insurability with other insurers.</t>
         </is>
       </c>
-      <c r="N5" s="4" t="inlineStr">
+      <c r="U5" s="4" t="inlineStr">
         <is>
           <t>DRN4969124.pdf</t>
         </is>
@@ -860,62 +1034,95 @@
           <t>DRN-4334761</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Royal &amp; Sun Alliance Insurance Ltd (RSA)</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>07 Dec 2023</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>Escape of water — loft pipe, unoccupied property, endorsement exclusion challenge</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Internal water pipe in loft of unoccupied property</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Unoccupied residential property</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
         <is>
           <t>Insurer declined under a policy endorsement that excluded damage caused by escape of water from 'any interior fixed heating or domestic water installation, washing machine or dishwasher'</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="K6" s="3" t="inlineStr">
         <is>
           <t>Customer disputed that a loft pipe built into the walls was a 'fixed installation' per the exclusion (distinguished from removable appliances like washing machines). Insurer argued endorsement was clearly laid out on the policy schedule. Broker claimed verbal disclosure at point of sale — no written evidence provided. FOS found the endorsement was not sufficiently highlighted in the Insurance Product Information document despite it listing a section specifically for restrictions.</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M6" s="3" t="inlineStr">
         <is>
           <t>Upheld — endorsement was a significant and unusual term that FCA guidance required to be clearly highlighted outside main policy terms. It was not sufficiently disclosed. RSA must assess claim without applying the endorsement, reimburse claim costs plus 8% simple interest, pay £150 compensation.</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="N6" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P6" s="3" t="inlineStr">
         <is>
           <t>FCA guidance requires significant and unusual exclusions to be clearly highlighted outside main policy terms (e.g. in IPID). IPID listed escape of water as a key inclusion with no mention of the restriction in the 'restrictions' section. Endorsement appeared on page 3 of policy schedule only.</t>
         </is>
       </c>
-      <c r="J6" s="3" t="inlineStr">
+      <c r="Q6" s="3" t="inlineStr">
         <is>
           <t>No written evidence from broker confirming the endorsement was specifically drawn to the customer's attention at point of sale. Only broker's own verbal recollection of a phone call provided.</t>
         </is>
       </c>
-      <c r="K6" s="3" t="inlineStr">
+      <c r="R6" s="3" t="inlineStr">
         <is>
           <t>The endorsement significantly restricted what is a standard and expected cover for an unoccupied property — escape of water is a primary risk for unoccupied properties. The IPID listed escape of water as covered but made no mention of the significant restriction in its 'restrictions' section. FCA guidance requires significant/unusual terms to be highlighted outside main policy terms. Broker's unsubstantiated verbal recollection was insufficient to prove adequate disclosure. Customer could not make an informed decision without clear disclosure. RSA responsible for ensuring its own documentation is adequate — cannot rely solely on broker's verbal assertion.</t>
         </is>
       </c>
-      <c r="L6" s="3" t="inlineStr">
+      <c r="S6" s="3" t="inlineStr">
         <is>
           <t>Significant endorsements restricting standard escape of water cover must appear prominently in the IPID restrictions section — presence in the policy schedule alone is insufficient. Unoccupied property policies frequently carry restrictive escape of water endorsements — always check and flag these specifically. Broker verbal disclosure without written evidence is insufficient to prove FCA disclosure obligations were met. FCA consumer duty and disclosure obligations are a primary challenge mechanism when insurer relies on an unusual exclusion.</t>
         </is>
       </c>
-      <c r="M6" s="3" t="inlineStr">
+      <c r="T6" s="3" t="inlineStr">
         <is>
           <t>If insurer relies on an endorsement to decline an escape of water claim: (1) check whether the endorsement appeared in the IPID restrictions section (not just policy schedule); (2) check whether written evidence of point-of-sale disclosure exists; (3) flag unoccupied property policies with escape of water endorsements as requiring explicit IPID disclosure check. If IPID does not mention the restriction, flag as potential FCA disclosure failure — assess claim without the endorsement.</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr">
+      <c r="U6" s="2" t="inlineStr">
         <is>
           <t>DRN-4334761.pdf</t>
         </is>
@@ -932,62 +1139,95 @@
           <t>DRN-1135035</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Covea Insurance plc</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>08 Apr 2020</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>Escape of water — lounge ceiling collapse, alleged leaking water tank</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>Alleged leaking water tank above lounge ceiling (insurer disputed — no moisture or staining found)</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="G7" s="4" t="inlineStr">
         <is>
           <t>Residential home</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
         <is>
           <t>Full decline — insurer's surveyor found no moisture or staining at damaged ceiling; concluded natural breakdown of 120-year-old plaster/lath ceiling materials (wear and tear), not caused by escape of water</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="K7" s="5" t="inlineStr">
         <is>
           <t>Plumber initially said leaking tank may have caused the collapse but provided no written report. Customer said ceiling was wet when it fell but had dried by the time surveyor attended (~3 weeks later). Surveyor conducted moisture tests and found no moisture present in the damaged area.</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M7" s="5" t="inlineStr">
         <is>
           <t>Not upheld — insurer's decision to decline was fair. Only expert written evidence available (surveyor's report) concluded damage was not due to escape of water. Customer did not obtain an independent expert report. Covea correctly declined.</t>
         </is>
       </c>
-      <c r="I7" s="5" t="inlineStr">
+      <c r="N7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P7" s="5" t="inlineStr">
         <is>
           <t>Coverage requires damage to be caused by a listed insured event. Wear and tear and gradual breakdown excluded. General Exclusions clause 13: loss or damage caused by wear and tear, wet or dry rot, or anything which happens gradually.</t>
         </is>
       </c>
-      <c r="J7" s="5" t="inlineStr">
+      <c r="Q7" s="5" t="inlineStr">
         <is>
           <t>No written report from initial plumber. No independent expert report obtained by customer. Fallen ceiling pieces disposed of before moisture testing.</t>
         </is>
       </c>
-      <c r="K7" s="5" t="inlineStr">
+      <c r="R7" s="5" t="inlineStr">
         <is>
           <t>Only expert written evidence available concluded damage was not due to escape of water. Natural breakdown of 120-year-old plaster and lath ceiling is consistent with gradual wear and tear. Delay before surveyor arrived was due to broker, not insurer. Customer had the opportunity to commission an independent expert report but did not do so.</t>
         </is>
       </c>
-      <c r="L7" s="5" t="inlineStr">
+      <c r="S7" s="5" t="inlineStr">
         <is>
           <t>A single plumber's unwritten verbal suggestion that a leak 'may have caused' damage is insufficient to establish escape of water. Surveyor moisture tests with no moisture detected are more persuasive than unsubstantiated claims. Customer who fails to obtain an independent expert report is at risk of losing a dispute where only the insurer's expert opinion exists.</t>
         </is>
       </c>
-      <c r="M7" s="5" t="inlineStr">
+      <c r="T7" s="5" t="inlineStr">
         <is>
           <t>If only insurer's expert opinion is available and customer has not obtained an independent report, treat decline as valid. Plumber's verbal suggestion without a written report is insufficient to establish escape of water. If customer claims damp dried before surveyor arrived, require contemporaneous evidence (photos, moisture readings).</t>
         </is>
       </c>
-      <c r="N7" s="4" t="inlineStr">
+      <c r="U7" s="4" t="inlineStr">
         <is>
           <t>DRN-1135035.pdf</t>
         </is>
@@ -1004,62 +1244,95 @@
           <t>DRN-1525346</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>AXA Insurance UK Plc</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>29 Jul 2020</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>Escape of water — secondary electrical failure claim; kitchen electrics attributed to 2018 hot water pipe escape</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>Mains hot water pipe in downstairs bathroom (2018 original incident; 2019 secondary electrical claim)</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Residential home</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
         <is>
           <t>Declined — insurer's engineer found a dead short in the circuit (mechanical cable break, not water-caused); kitchen was on a separate electrical ring barely affected by the original escape; 7-month delay between original escape and electrical failure makes water causation implausible</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="K8" s="3" t="inlineStr">
         <is>
           <t>Customer argued steam from hot water pipe spread through the property and damaged the consumer unit and kitchen electrics. Customer's own 2018 electrician report recommended work on the consumer unit. AXA's engineer tested the circuit and found a dead short (mechanical cable break, not water-related). Kitchen was on a different ring to the rest of the property and showed only minor aesthetic damage from the original escape.</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
         <is>
           <t>Not upheld — AXA's decision to decline was fair. Dead short is a mechanical cable failure, not caused by water. Kitchen was on a separate electrical ring and barely affected by the original escape. Customer's 2018 electrician report related to the consumer unit, not the circuit fault causing the 2019 failure.</t>
         </is>
       </c>
-      <c r="I8" s="3" t="inlineStr">
+      <c r="N8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P8" s="3" t="inlineStr">
         <is>
           <t>Coverage requires damage to have been caused by an insured peril. If electrical failure was caused by a maintenance problem (dead short — mechanical fault), there is no insured peril and no cover applies.</t>
         </is>
       </c>
-      <c r="J8" s="3" t="inlineStr">
+      <c r="Q8" s="3" t="inlineStr">
         <is>
           <t>No independent electrician's report specifically addressing the 2019 fault type (dead short vs. water damage). Customer's 2018 report related to consumer unit only, not the circuit.</t>
         </is>
       </c>
-      <c r="K8" s="3" t="inlineStr">
+      <c r="R8" s="3" t="inlineStr">
         <is>
           <t>AXA's engineer found a dead short (mechanical break in cable), which cannot be caused by water. Kitchen was on a separate electrical ring from the rest of the property and barely affected by the original escape of water. Seven-month delay between original escape and electrical failure makes water causation unlikely. Customer's 2018 electrician report did not address the specific circuit fault causing the 2019 failure.</t>
         </is>
       </c>
-      <c r="L8" s="3" t="inlineStr">
+      <c r="S8" s="3" t="inlineStr">
         <is>
           <t>Delayed secondary claims for electrical failure following an escape of water require evidence that the fault was caused by water, not mechanical failure. A dead short in a circuit is a distinct mechanical fault not caused by water. Insurer's expert report on the specific fault type is more persuasive than a general report about the consumer unit. Time elapsed between escape of water and reported electrical failure is relevant to causation assessment.</t>
         </is>
       </c>
-      <c r="M8" s="3" t="inlineStr">
+      <c r="T8" s="3" t="inlineStr">
         <is>
           <t>For secondary electrical claims following escape of water: require independent electrical inspection report addressing the specific fault type. If insurer's expert finds fault is mechanical (dead short, cable break) and customer provides no contradicting expert report, decline on maintenance grounds. 7+ months elapsed between escape of water and electrical failure is a negative indicator for water causation.</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="U8" s="2" t="inlineStr">
         <is>
           <t>DRN-1525346.pdf</t>
         </is>
@@ -1076,62 +1349,95 @@
           <t>DRN-1623377</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Insurers at Lloyd's (Society of Lloyd's)</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>06 May 2020</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>Escape of water — attic pipe failure in unoccupied property; Structural Works Clause endorsement applied from policy inception</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="F9" s="5" t="inlineStr">
         <is>
           <t>Attic pipe (elbow joint failure) in unoccupied property intended for future refurbishment</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="G9" s="4" t="inlineStr">
         <is>
           <t>Unoccupied residential property (intended for refurbishment)</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J9" s="5" t="inlineStr">
         <is>
           <t>Full decline — Structural Works Clause endorsement excluded escape of water cover until all disclosed structural work was fully completed; endorsement applied from policy inception regardless of whether works had yet started</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="K9" s="5" t="inlineStr">
         <is>
           <t>Customer argued the endorsement should not apply because structural works had not yet started. Insurer maintained the endorsement applied from inception, regardless of whether works had started. Loss adjuster's preliminary report left open whether the heating clause was complied with and identified the cause as an elbow joint failure — but insurer's final coverage decision rested on the endorsement.</t>
         </is>
       </c>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="L9" s="4" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M9" s="5" t="inlineStr">
         <is>
           <t>Not upheld — policy wording was clear. Endorsement applied at all times and from inception. Customer's own disclosure of intended structural works at inception triggered the clause. Loss adjuster's preliminary assessment did not override insurer's final coverage decision.</t>
         </is>
       </c>
-      <c r="I9" s="5" t="inlineStr">
+      <c r="N9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P9" s="5" t="inlineStr">
         <is>
           <t>Structural Works Clause endorsement: 'This insurance does not provide cover for Escape of Water or Trace and Access until all the structural work, as disclosed to us, has been fully completed.' Schedule stated endorsements apply 'at all times.'</t>
         </is>
       </c>
-      <c r="J9" s="5" t="inlineStr">
+      <c r="Q9" s="5" t="inlineStr">
         <is>
           <t>No written confirmation from loss adjuster that heating clause was complied with (not decisive given endorsement applied regardless). No definitive cause report from plumber on elbow joint failure.</t>
         </is>
       </c>
-      <c r="K9" s="5" t="inlineStr">
+      <c r="R9" s="5" t="inlineStr">
         <is>
           <t>Schedule of Cover stated all endorsements apply 'at all times.' The Structural Works Clause clearly excluded escape of water until structural works were fully completed. Customer's own disclosure of intended works at inception triggered the endorsement from day one. Endorsement wording was unambiguous. Loss adjuster's preliminary views were not binding on the insurer.</t>
         </is>
       </c>
-      <c r="L9" s="5" t="inlineStr">
+      <c r="S9" s="5" t="inlineStr">
         <is>
           <t>Structural Works Clause endorsements on unoccupied properties exclude escape of water from policy inception — the works do not need to have started. Insurer's policy documentation controls the coverage decision; loss adjuster's preliminary on-site views are not determinative. Customer disclosure of intended structural works at inception triggers the endorsement immediately.</t>
         </is>
       </c>
-      <c r="M9" s="5" t="inlineStr">
+      <c r="T9" s="5" t="inlineStr">
         <is>
           <t>On unoccupied property escape of water claims: always check for Structural Works Clause endorsement. If present and disclosed works have not been fully completed, apply endorsement to decline regardless of whether works have started. Loss adjuster's preliminary views are not binding on insurer's final coverage decision.</t>
         </is>
       </c>
-      <c r="N9" s="4" t="inlineStr">
+      <c r="U9" s="4" t="inlineStr">
         <is>
           <t>DRN-1623377.pdf</t>
         </is>
@@ -1148,62 +1454,95 @@
           <t>DRN-2340952</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>U K Insurance Limited (UKI)</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>10 Mar 2021</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>Escape of water — accepted claim; disputed handling: scope of reinstatement, quality of works, individual items (cooker, bed, electrics, boiler, drying), and adequacy of compensation</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
+      <c r="F10" s="3" t="inlineStr">
         <is>
           <t>Escape of water affecting bathroom, kitchen and spare room</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Residential home</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>Handling / Reinstatement Dispute</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Accepted — Disputed Settlement</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
         <is>
           <t>Not a coverage rejection — claim accepted. Individual items declined: cooker and boiler (no causation evidence); electrical safety (pre-existing wiring issues unrelated to escape); loss of rent (no evidence of prior rental intention); bed (no evidence contractor damaged it). Total £750 compensation offered (£350 + £400).</t>
         </is>
       </c>
-      <c r="G10" s="3" t="inlineStr">
+      <c r="K10" s="3" t="inlineStr">
         <is>
           <t>Customer disputed: kitchen tiling gap (caused by customer-chosen layout change, not insurer); quality of repairs; cooker damage (no expert evidence linking to escape of water); bed removed by contractor in error; electrical safety post-repair; adequacy of drying (drying certificate issued); boiler damage (no evidence); loss of rental income from spare room.</t>
         </is>
       </c>
-      <c r="H10" s="3" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M10" s="3" t="inlineStr">
         <is>
           <t>Not upheld — revised cash settlement (£1,086 buildings + £700 contents) was fair. Individual item disputes rejected for lack of causation evidence. £750 total compensation was fair given some delays were partly due to customer's unavailability. Insurer's revised calculation correcting an earlier error was accepted.</t>
         </is>
       </c>
-      <c r="I10" s="3" t="inlineStr">
+      <c r="N10" s="2" t="n">
+        <v>750</v>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>No — Handling Dispute</t>
+        </is>
+      </c>
+      <c r="P10" s="3" t="inlineStr">
         <is>
           <t>Insurer obligated to reinstate damage caused by escape of water. Items must be shown to have been damaged by the escape of water. Policy excess applies.</t>
         </is>
       </c>
-      <c r="J10" s="3" t="inlineStr">
+      <c r="Q10" s="3" t="inlineStr">
         <is>
           <t>No expert evidence linking cooker, boiler, or electrics to escape of water. No evidence of pre-rental intention for spare room before March 2020. No evidence property was not properly dried (drying certificate accepted). No photographic evidence contractor damaged the bed.</t>
         </is>
       </c>
-      <c r="K10" s="3" t="inlineStr">
+      <c r="R10" s="3" t="inlineStr">
         <is>
           <t>Cash settlement methodology was fair once insurer corrected calculation error. Scope disputes resolved in insurer's favour. Each individual item dispute required specific causation evidence which customer could not provide. Customer-caused delays (unavailability) reduced compensation entitlement. Drying certificate issued by contractor was accepted as evidence of completed drying.</t>
         </is>
       </c>
-      <c r="L10" s="3" t="inlineStr">
+      <c r="S10" s="3" t="inlineStr">
         <is>
           <t>Claims handling disputes require item-by-item causation evidence linking each disputed item to the escape of water. Insurer should correct calculation errors promptly. Customer-caused delays (unavailability, refusal of access) mitigate compensation quantum. A drying certificate from insurer's contractor is presumptive evidence of completed drying unless contradicted by independent expert evidence.</t>
         </is>
       </c>
-      <c r="M10" s="3" t="inlineStr">
+      <c r="T10" s="3" t="inlineStr">
         <is>
           <t>For each item in a disputed claim, require specific expert causation evidence linking it to the escape of water. Accept insurer's revised cash settlement if methodology is fair. Flag customer-caused delays as a mitigating factor in compensation assessment. Drying certificate from insurer's contractor is presumptive evidence of completed drying — rebuttable only by independent expert report.</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="U10" s="2" t="inlineStr">
         <is>
           <t>DRN-2340952.pdf</t>
         </is>
@@ -1220,62 +1559,95 @@
           <t>DRN2512341</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Zurich Insurance PLC</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>28 Feb 2019</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
         <is>
           <t>Escape of water — pre-policy wet rot damage to floor joists; customer sought to invoke secondary flooding industry approach</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="F11" s="5" t="inlineStr">
         <is>
           <t>Wet rot in floor joists under two bedrooms — attributed to previous owner's prior 'serious flood' (determined to be likely escape of water, not a natural flood)</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="G11" s="4" t="inlineStr">
         <is>
           <t>Residential home (recently purchased)</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>Pre-Inception Damage Dispute</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
         <is>
           <t>Full decline — damage predated policy inception; secondary flooding industry approach does not apply because original cause was escape of water, not a natural flood; current insurer only liable for damage occurring after policy start date</t>
         </is>
       </c>
-      <c r="G11" s="5" t="inlineStr">
+      <c r="K11" s="5" t="inlineStr">
         <is>
           <t>Customer argued original incident was 'secondary flooding' per FOS technical note. FOS distinguished natural flood from escape of water — escape of water does not trigger secondary flooding policy. Customer later argued property was in a surface water flooding risk area and found water in the floor void during recent renovations, suggesting possible natural flood origin.</t>
         </is>
       </c>
-      <c r="H11" s="5" t="inlineStr">
+      <c r="L11" s="4" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M11" s="5" t="inlineStr">
         <is>
           <t>Not upheld — Zurich's decline was fair. No persuasive evidence the original cause was a natural flood rather than an escape of water. Secondary flooding industry approach requires confirmed natural flood cause. Customer's later evidence (surface water flood risk area, water in void) was speculative and insufficient.</t>
         </is>
       </c>
-      <c r="I11" s="5" t="inlineStr">
+      <c r="N11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P11" s="5" t="inlineStr">
         <is>
           <t>Policy covers damage during the period of insurance only. Existing damage exclusion. Secondary flooding industry agreement applies only where original cause was a natural flood — escape of water, even if it causes flooding of the property, does not qualify.</t>
         </is>
       </c>
-      <c r="J11" s="5" t="inlineStr">
+      <c r="Q11" s="5" t="inlineStr">
         <is>
           <t>Original claim file not available. No documentary evidence original cause was a natural flood. No evidence prior insurer treated the claim as flood rather than escape of water.</t>
         </is>
       </c>
-      <c r="K11" s="5" t="inlineStr">
+      <c r="R11" s="5" t="inlineStr">
         <is>
           <t>Secondary flooding industry approach applies only to natural flood events. An escape of water, even if it floods a property, remains an escape of water event. Customer's original characterisation (escape of water) was partly their own speculation. No persuasive evidence the original incident was a natural flood. Customer's later surface water flooding argument was speculative — nothing linked the floor void water to the original damage.</t>
         </is>
       </c>
-      <c r="L11" s="5" t="inlineStr">
+      <c r="S11" s="5" t="inlineStr">
         <is>
           <t>Secondary flooding industry approach does not apply where original cause was escape of water. Current insurer is not responsible for damage preceding policy inception. Absence of original claim file is an evidential gap against the policyholder. Customer speculation about original cause is insufficient — documentary evidence of the original claim and its cause is required.</t>
         </is>
       </c>
-      <c r="M11" s="5" t="inlineStr">
+      <c r="T11" s="5" t="inlineStr">
         <is>
           <t>For claims where damage predates policy inception: reject unless secondary flooding industry agreement applies (requires confirmed natural flood cause with documentary evidence). Do not apply secondary flooding approach where original cause was escape of water. Require original claim file or insurer records showing original event was treated as flood before applying secondary flooding.</t>
         </is>
       </c>
-      <c r="N11" s="4" t="inlineStr">
+      <c r="U11" s="4" t="inlineStr">
         <is>
           <t>DRN2512341.pdf</t>
         </is>
@@ -1292,62 +1664,95 @@
           <t>DRN-2540997</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Fairmead Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>01 Mar 2021</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
         <is>
           <t>Escape of water — two pre-existing damage claims discovered shortly after purchase (kitchen floor and bathroom floor)</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>Kitchen: escape of water from kitchen services (historic); Bathroom: pipe connecting WC to cistern (historic)</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Residential home (recently purchased)</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>Pre-Inception Damage Dispute</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
         <is>
           <t>Both claims declined — insurer concluded damage occurred before policy inception and/or was caused gradually. Loss adjuster assessed kitchen only; no assessment of bathroom.</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr">
+      <c r="K12" s="3" t="inlineStr">
         <is>
           <t>Customer commissioned a full pre-purchase structural survey which found no flooring issues. Damage not discovered until weeks after moving in. Specialist leak detection found no active leaks (damage historic). Insurer's loss adjuster assessed kitchen but not bathroom. Insurer's call handler implied claims would be covered — no written record.</t>
         </is>
       </c>
-      <c r="H12" s="3" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M12" s="3" t="inlineStr">
         <is>
           <t>Upheld — Fairmead must accept both claims. Pay restoration costs already incurred plus 8% simple interest. Pay trace and access costs. Settle remaining uninstructed work using insurer's contractors or equivalent cost. £400 compensation. Applying pre-existing or gradual exclusion was unfair — customer could not reasonably have known about damage; full structural survey found nothing; damage was fully concealed.</t>
         </is>
       </c>
-      <c r="I12" s="3" t="inlineStr">
+      <c r="N12" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P12" s="3" t="inlineStr">
         <is>
           <t>Pre-existing damage exclusion; gradual damage exclusion. FOS approach: applying gradual damage exclusion is unfair if consumer could not reasonably have been aware of damage occurring. Policy covers escape of water and buildings including wooden, laminate and vinyl floor coverings.</t>
         </is>
       </c>
-      <c r="J12" s="3" t="inlineStr">
+      <c r="Q12" s="3" t="inlineStr">
         <is>
           <t>No active leaks at time of survey (historic damage). No written record of call handler implying coverage. No evidence prior owners or surveyors were aware of the damage.</t>
         </is>
       </c>
-      <c r="K12" s="3" t="inlineStr">
+      <c r="R12" s="3" t="inlineStr">
         <is>
           <t>Pre-purchase structural survey found no flooring issues — no one (including prior owners or surveyors) would have known about the damage. Customer discovered problems within weeks of moving in. Applying pre-existing exclusion is unfair where customer had no reasonable means of discovering the damage. Gradual damage exclusion equally unfair — customer did not live at property when damage occurred and was prevented from noticing it. Insurer must assess all claimed areas, not just kitchen.</t>
         </is>
       </c>
-      <c r="L12" s="3" t="inlineStr">
+      <c r="S12" s="3" t="inlineStr">
         <is>
           <t>If customer commissioned a pre-purchase structural survey that identified no issues and damage was discovered shortly after moving in, it is unfair to apply pre-existing or gradual damage exclusions — customer could not reasonably have known. Insurer must assess all claimed areas; sending loss adjuster to kitchen only and ignoring bathroom is an incomplete assessment.</t>
         </is>
       </c>
-      <c r="M12" s="3" t="inlineStr">
+      <c r="T12" s="3" t="inlineStr">
         <is>
           <t>If pre-existing or gradual damage exclusion is applied but customer commissioned a pre-purchase structural survey finding no issues, and damage was discovered shortly after moving in: reject exclusion application as unfair — customer could not reasonably have known. Insurer must assess all claimed rooms. Pay trace and access as standalone benefit where applicable.</t>
         </is>
       </c>
-      <c r="N12" s="2" t="inlineStr">
+      <c r="U12" s="2" t="inlineStr">
         <is>
           <t>DRN-2540997.pdf</t>
         </is>
@@ -1364,62 +1769,95 @@
           <t>DRN-2572816</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Admiral Insurance (Gibraltar) Limited</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>20 Apr 2021</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
         <is>
           <t>Escape of water — leaking drain pipe under kitchen floor causing dry rot in floor joists; insurer invoked gradually operating cause and faulty design (ventilation) exclusions</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="F13" s="5" t="inlineStr">
         <is>
           <t>Leaking drain pipe under kitchen floor</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="G13" s="4" t="inlineStr">
         <is>
           <t>Residential home (kitchen)</t>
         </is>
       </c>
-      <c r="F13" s="5" t="inlineStr">
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J13" s="5" t="inlineStr">
         <is>
           <t>Declined — gradually operating cause (dry rot developed over time and not linked to escape of water); faulty design exclusion (kitchen extension allegedly lacked proper ventilation). Insurer offered £100 compensation for poor service only.</t>
         </is>
       </c>
-      <c r="G13" s="5" t="inlineStr">
+      <c r="K13" s="5" t="inlineStr">
         <is>
           <t>Insurer's second expert concluded dry rot developed over time but drew no link between the leaking drain in the same area and the dry rot. Insurer's own restoration schedule listed cause as 'escape of water.' Phone call between insurer and contractor acknowledged the leak likely caused the dry rot. Insurer provided no evidence of ventilation requirements or building regulations to support faulty design exclusion.</t>
         </is>
       </c>
-      <c r="H13" s="5" t="inlineStr">
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M13" s="5" t="inlineStr">
         <is>
           <t>Upheld — Admiral failed to prove either exclusion applies. Must accept claim under escape of water peril and settle in line with policy terms. Additional £300 compensation (total £400 including £100 already paid).</t>
         </is>
       </c>
-      <c r="I13" s="5" t="inlineStr">
+      <c r="N13" s="4" t="n">
+        <v>400</v>
+      </c>
+      <c r="O13" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P13" s="5" t="inlineStr">
         <is>
           <t>Gradually operating cause exclusion; faulty design exclusion. Once insured peril established (escape of water accepted), insurer must prove exclusion applies with specific evidence. Insurer cannot merely assert exclusion.</t>
         </is>
       </c>
-      <c r="J13" s="5" t="inlineStr">
+      <c r="Q13" s="5" t="inlineStr">
         <is>
           <t>No reasoning in insurer's expert report why dry rot was unrelated to the leaking drain in the same area. No building regulations or ventilation standards cited to support faulty design exclusion.</t>
         </is>
       </c>
-      <c r="K13" s="5" t="inlineStr">
+      <c r="R13" s="5" t="inlineStr">
         <is>
           <t>Insurer accepted escape of water as the insured peril but declined on exclusions. Second expert report drew no causal link between the leaking drain and the dry rot — the conclusion 'unrelated' was offered with no reasoning. Dry rot develops on damp timber; a leaking drain in the same area makes the link obvious. Insurer's own restoration schedule listed cause as escape of water. Phone call with contractor confirmed insurer's acceptance of the link. No evidence provided for the ventilation/faulty design exclusion. Concealed damage under floor — customer could not reasonably have been aware.</t>
         </is>
       </c>
-      <c r="L13" s="5" t="inlineStr">
+      <c r="S13" s="5" t="inlineStr">
         <is>
           <t>When insurer relies on gradually operating cause or faulty design exclusion, it must provide specific evidence proving the exclusion — not just assert it. Insurer's own internal records (restoration schedules, contractor call notes) acknowledging escape of water as the cause are binding admissions. Dry rot in proximity to a leaking pipe does not prove independence from the leak. Concealed pipe leak under floor: customer had no reasonable opportunity to be aware of damage developing.</t>
         </is>
       </c>
-      <c r="M13" s="5" t="inlineStr">
+      <c r="T13" s="5" t="inlineStr">
         <is>
           <t>If insurer relies on gradually operating cause or faulty design exclusion: require specific evidence proving the exclusion (cause analysis; building regulations for ventilation claim). If insurer's own documents reference escape of water as cause, treat as binding admissions. Where dry rot is found proximate to a confirmed leaking pipe, insurer must prove dry rot was independent of the escape of water. Flag concealed pipe leaks under floors as circumstances where gradual damage exclusion should not automatically apply.</t>
         </is>
       </c>
-      <c r="N13" s="4" t="inlineStr">
+      <c r="U13" s="4" t="inlineStr">
         <is>
           <t>DRN-2572816.pdf</t>
         </is>
@@ -1436,62 +1874,95 @@
           <t>DRN-2749125</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Covea Insurance Plc</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>29 Jun 2021</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
         <is>
           <t>Escape of water — perished copper pipe, slow constant leak under kitchen floor, discovered when new appliance installed</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="F14" s="3" t="inlineStr">
         <is>
           <t>Perished copper pipe causing slow constant leak under kitchen floor</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>Residential home (kitchen)</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>Pre-Inception Damage Dispute</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
         <is>
           <t>Claim declined — insurer concluded damage predated policy inception (October 2019); insurer's buildings inspector's 28-page report with time-stamped photographs showed severely rotten floorboards and joists consistent with multi-year leaking</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr">
+      <c r="K14" s="3" t="inlineStr">
         <is>
           <t>Customer stated they commissioned a structural survey before purchase (2014) which found no issues. Customer had a new kitchen professionally installed a few years prior with no visible leak. Customer was first alerted to damage in July 2020 when a new washing machine was being fitted. Insurer's buildings inspector produced a detailed 28-page report with time-stamped photos — customer disputed inspector spent only 5 minutes at the property.</t>
         </is>
       </c>
-      <c r="H14" s="3" t="inlineStr">
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>Compensation Only</t>
+        </is>
+      </c>
+      <c r="M14" s="3" t="inlineStr">
         <is>
           <t>Upheld in part — coverage decline upheld (damage predated policy inception; severely rotten floorboards consistent with multi-year leaking; visible signs of structural degradation — dropping kitchen units and worktop — meant customer ought reasonably to have been aware). Covea must pay £200 compensation for avoidable delays (approximately one month from report to repudiation).</t>
         </is>
       </c>
-      <c r="I14" s="3" t="inlineStr">
+      <c r="N14" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P14" s="3" t="inlineStr">
         <is>
           <t>Pre-existing damage exclusion; gradually operating cause exclusion; wet or dry rot exclusion. Damage must occur after policy inception. Gradual damage exclusion applies where customer ought reasonably to have been aware of damage occurring.</t>
         </is>
       </c>
-      <c r="J14" s="3" t="inlineStr">
+      <c r="Q14" s="3" t="inlineStr">
         <is>
           <t>No evidence floorboards were inspected and damage-free during kitchen refurbishment. Structural survey did not assess under-floor condition adequately. No evidence from prior insurer covering period of alleged deterioration.</t>
         </is>
       </c>
-      <c r="K14" s="3" t="inlineStr">
+      <c r="R14" s="3" t="inlineStr">
         <is>
           <t>Buildings inspector's 28-page report with time-stamped photographs was detailed and persuasive. Severely rotten floorboards and joists consistent with multi-year leaking — damage unlikely to have originated after October 2019 inception. Dropping kitchen units and worktop were visible signs of structural degradation — customer ought reasonably to have been aware earlier. This distinguishes the case from EOW-011 (DRN-2540997) where damage was fully concealed with no visible signs.</t>
         </is>
       </c>
-      <c r="L14" s="3" t="inlineStr">
+      <c r="S14" s="3" t="inlineStr">
         <is>
           <t>A detailed buildings inspector report with time-stamped photographs showing multi-year deterioration is highly persuasive evidence of pre-inception damage. Visible signs of structural degradation (dropping units, sinking worktop) represent a reasonable opportunity for the customer to have investigated earlier. Contrasts with EOW-011 (DRN-2540997) where damage was fully concealed and no visible indicators existed. Always compensate for avoidable claim processing delays even where coverage is correctly declined.</t>
         </is>
       </c>
-      <c r="M14" s="3" t="inlineStr">
+      <c r="T14" s="3" t="inlineStr">
         <is>
           <t>Where insurer provides a detailed inspector report (with time-stamped photos) showing damage consistent with multi-year gradual deterioration, support pre-existing decline. Where visible signs of degradation existed (dropping units, sinking surfaces), customer ought reasonably to have been aware — uphold gradual exclusion. Differentiate from cases where damage is fully concealed with no visible indicators (see EOW-011). Compensate for avoidable delays regardless of coverage outcome.</t>
         </is>
       </c>
-      <c r="N14" s="2" t="inlineStr">
+      <c r="U14" s="2" t="inlineStr">
         <is>
           <t>DRN-2749125.pdf</t>
         </is>
@@ -1508,62 +1979,95 @@
           <t>DRN-2771304</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>AXA Insurance UK Plc</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>20 May 2021</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
         <is>
           <t>Escape of water — peril classification dispute; tap left on by resident causing water damage to managed flats; AXA applied £5,000 escape of water excess instead of £250 damage excess</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="F15" s="5" t="inlineStr">
         <is>
           <t>Tap left on by a resident in a managed flat (human negligence / overflow, not a pipe failure)</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="G15" s="4" t="inlineStr">
         <is>
           <t>Commercial / Management Company</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>Peril Classification Dispute</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>Accepted — Disputed Settlement</t>
+        </is>
+      </c>
+      <c r="J15" s="5" t="inlineStr">
         <is>
           <t>Not a coverage rejection — AXA accepted the claim but misclassified it under the escape of water peril (£5,000 excess) rather than as accidental damage or general damage (£250 excess). Dispute was solely about peril classification and applicable excess.</t>
         </is>
       </c>
-      <c r="G15" s="5" t="inlineStr">
+      <c r="K15" s="5" t="inlineStr">
         <is>
           <t>Insurer maintained tap-left-on = escape of water (£5,000 excess). Management company argued it was accidental damage (£250 excess). FOS reviewed multiple standard insurer policies — tap-left-on is typically classified as accidental damage, not escape of water. AXA submitted a prior adjudicator view classifying tap-left-on as escape of water, but ombudsman did not follow it.</t>
         </is>
       </c>
-      <c r="H15" s="5" t="inlineStr">
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M15" s="5" t="inlineStr">
         <is>
           <t>Upheld — claim should be classified as 'damage' (or accidental damage if insurer wishes to classify further), not escape of water. Lower excess to apply. £150 compensation for delays and inconvenience to flat owners and residents.</t>
         </is>
       </c>
-      <c r="I15" s="5" t="inlineStr">
+      <c r="N15" s="4" t="n">
+        <v>150</v>
+      </c>
+      <c r="O15" s="4" t="inlineStr">
+        <is>
+          <t>No — Commercial</t>
+        </is>
+      </c>
+      <c r="P15" s="5" t="inlineStr">
         <is>
           <t>All-risks policy covers 'damage' unless excluded. Escape of water excess endorsement (£5,000). Industry convention: tap-left-on = accidental damage, not escape of water. Correct peril classification is required to apply the correct excess.</t>
         </is>
       </c>
-      <c r="J15" s="5" t="inlineStr">
+      <c r="Q15" s="5" t="inlineStr">
         <is>
           <t>No standard industry examples found where tap-left-on is classified as escape of water.</t>
         </is>
       </c>
-      <c r="K15" s="5" t="inlineStr">
+      <c r="R15" s="5" t="inlineStr">
         <is>
           <t>Multiple standard insurer policies cover tap-left-on under accidental damage, not escape of water. No examples found where standard policies classify tap-left-on as escape of water. All-risks policy covers damage unless excluded — no relevant exclusion applied. Prior adjudicator view on a different case was not persuasive on the individual facts here. Incorrect classification causing higher excess deduction is a service failure.</t>
         </is>
       </c>
-      <c r="L15" s="5" t="inlineStr">
+      <c r="S15" s="5" t="inlineStr">
         <is>
           <t>Tap-left-on incidents should be classified as accidental damage, not escape of water, when policy contains separate excess structures. On all-risks policies, classify as 'damage' unless a specific exclusion applies. Incorrect peril classification causing a higher excess deduction is a service failure warranting compensation. NOTE: This case involves a commercial all-risks policy for a managed residential block — classification rules derived here may not apply directly to standard residential home insurance policies.</t>
         </is>
       </c>
-      <c r="M15" s="5" t="inlineStr">
+      <c r="T15" s="5" t="inlineStr">
         <is>
           <t>Water damage caused by a tap being left on: classify as accidental damage (not escape of water) when policy contains separate excess structures for each peril. Do not apply escape of water excess to tap-left-on incidents. On all-risks policies, classify as 'damage' unless a specific exclusion prevents it. Note: rule derived from commercial all-risks context — verify applicability before applying to standard residential policies.</t>
         </is>
       </c>
-      <c r="N15" s="4" t="inlineStr">
+      <c r="U15" s="4" t="inlineStr">
         <is>
           <t>DRN-2771304.pdf</t>
         </is>
@@ -1580,62 +2084,95 @@
           <t>DRN-2806638</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Endsleigh Insurance Services Ltd</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>01 Jul 2021</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
         <is>
           <t>Broker Disclosure Dispute</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="F16" s="3" t="inlineStr">
         <is>
           <t>Broken toilet cistern causing floor damage</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>Leasehold flat (property owners policy — lessee and management company director)</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>Broker Conduct Dispute</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
         <is>
           <t>Not a coverage rejection — claim was paid. Dispute was whether broker (Endsleigh) adequately disclosed that the escape of water excess had increased from £200 to £500 at 2019 renewal, resulting in policyholder receiving £300 less settlement than expected.</t>
         </is>
       </c>
-      <c r="G16" s="3" t="inlineStr">
+      <c r="K16" s="3" t="inlineStr">
         <is>
           <t>Policyholder accepted excess increase was communicated in 2019 renewal documents but argued 2020 renewal documents did not link excess levels (A/B/C) to specific perils. Broker confirmed it had notified insurer that 2020 documents lacked this mapping — but this was outside the scope of the 2019 renewal complaint before FOS.</t>
         </is>
       </c>
-      <c r="H16" s="3" t="inlineStr">
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M16" s="3" t="inlineStr">
         <is>
           <t>Not upheld (2019 renewal complaint) — excess increase was clearly communicated across multiple 2019 renewal documents; policyholder accepted renewal and paid premium. 2020 renewal document clarity issue is a separate complaint, not within scope of this FOS referral.</t>
         </is>
       </c>
-      <c r="I16" s="3" t="inlineStr">
+      <c r="N16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>No — Broker Dispute</t>
+        </is>
+      </c>
+      <c r="P16" s="3" t="inlineStr">
         <is>
           <t>Broker's duty to clearly disclose material policy changes at renewal. Escape of water excess endorsement increased from £200 to £500. Policyholder acceptance of renewal after clear disclosure binds them to the new terms. FOS can only review the complaint as originally submitted to the firm.</t>
         </is>
       </c>
-      <c r="J16" s="3" t="inlineStr">
+      <c r="Q16" s="3" t="inlineStr">
         <is>
           <t>2020 renewal documents failed to link each excess level (A/B/C) to the specific peril it applied to — but this was a separate complaint outside this referral scope.</t>
         </is>
       </c>
-      <c r="K16" s="3" t="inlineStr">
+      <c r="R16" s="3" t="inlineStr">
         <is>
           <t>Excess increase was communicated in multiple 2019 renewal documents (renewal invitation, statement of fact, schedule, Notice to Policyholder). Policyholder accepted renewal by paying premium — bound by new excess. Only the 2019 notification complaint was within scope. The 2020 document clarity issue must first be raised as a new complaint with the broker before FOS referral.</t>
         </is>
       </c>
-      <c r="L16" s="3" t="inlineStr">
+      <c r="S16" s="3" t="inlineStr">
         <is>
           <t>[NON-CORE — Broker Disclosure Dispute] Broker must clearly disclose material policy changes at renewal, preferably across multiple documents. Policyholder who pays premium after disclosure is bound by the new terms. Excess-to-peril mapping in renewal documents must be explicit — failure to link excess levels to specific perils in subsequent renewal years is a separate documentation complaint that must be raised with the broker first. This case concerns broker regulatory conduct, not claim assessment — flag as Non-Core for playbook development.</t>
         </is>
       </c>
-      <c r="M16" s="3" t="inlineStr">
+      <c r="T16" s="3" t="inlineStr">
         <is>
           <t>Excess increases at renewal: verify disclosure appears explicitly in multiple renewal documents. If policyholder paid premium and renewed after clear disclosure, apply the new excess. If renewal documents fail to link excess levels to specific perils, flag as potential documentation failure — but this is a separate complaint for the renewal year in which it first arose. [NON-CORE — broker conduct rule; not applicable to standard claim assessment playbook.]</t>
         </is>
       </c>
-      <c r="N16" s="2" t="inlineStr">
+      <c r="U16" s="2" t="inlineStr">
         <is>
           <t>DRN-2806638.pdf</t>
         </is>

</xml_diff>

<commit_message>
Add EOW-016 to EOW-025 to Escape of Water Case Database
</commit_message>
<xml_diff>
--- a/knowledge/case-databases/Escape_of_Water_Case_Database.xlsx
+++ b/knowledge/case-databases/Escape_of_Water_Case_Database.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U16"/>
+  <dimension ref="A1:U26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2178,6 +2178,1056 @@
         </is>
       </c>
     </row>
+    <row r="17" ht="120" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>EOW-016</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>DRN-3022853</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Admiral Insurance (Gibraltar) Limited</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>6 Jan 2022</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>Burst pipe in bathroom caused water damage to bathroom and kitchen below; dispute over settlement quantum with insurer attributing most claimed items to wear and tear rather than EOW</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>Burst pipe in bathroom</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I17" s="4" t="inlineStr">
+        <is>
+          <t>Accepted — Disputed Settlement</t>
+        </is>
+      </c>
+      <c r="J17" s="5" t="inlineStr">
+        <is>
+          <t>Independent surveyor assessed only £1,800 of damage attributable to EOW; remaining items in policyholder's £22,000 quote attributed to wear and tear and betterment</t>
+        </is>
+      </c>
+      <c r="K17" s="5" t="inlineStr">
+        <is>
+          <t>Policyholder relied on own tradesman quotes (~£22,000) and submitted video footage; insurer relied on detailed independent surveyor's report itemising each element and its cause</t>
+        </is>
+      </c>
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M17" s="5" t="inlineStr">
+        <is>
+          <t>FOS did not require Admiral to increase settlement beyond £1,200 offered (£1,800 assessed EOW damage less £600 excess); Admiral's surveyor-based assessment held to be reasonable and properly evidenced</t>
+        </is>
+      </c>
+      <c r="N17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P17" s="5" t="inlineStr">
+        <is>
+          <t>Policy covers damage caused by EOW only; wear and tear and betterment are excluded; insurer entitled to scope attributable damage using independent surveyor; settlement must restore policyholder to pre-loss position without improvement</t>
+        </is>
+      </c>
+      <c r="Q17" s="5" t="inlineStr">
+        <is>
+          <t>No independent counter-survey submitted by policyholder; videos submitted but did not establish additional EOW-attributable damage</t>
+        </is>
+      </c>
+      <c r="R17" s="5" t="inlineStr">
+        <is>
+          <t>FOS cannot make independent technical assessments; assessed whether insurer's process was reasonable; commissioning a detailed survey in response to an unusually high quote was proportionate; insurer reviewed its position when new evidence (videos) was submitted — process was fair</t>
+        </is>
+      </c>
+      <c r="S17" s="5" t="inlineStr">
+        <is>
+          <t>When policyholder quotes significantly exceed insurer's assessment, insurer may commission an independent survey to distinguish EOW damage from wear and tear; a well-evidenced surveyor's report is sufficient basis for a reduced settlement; FOS will not substitute its own technical judgment</t>
+        </is>
+      </c>
+      <c r="T17" s="5" t="inlineStr">
+        <is>
+          <t>IF settlement_disputed AND insurer_has_detailed_surveyor_report AND report_identifies_wear_and_tear_separately THEN surveyor_based_settlement IS defensible AND FOS_likely = Not_Upheld</t>
+        </is>
+      </c>
+      <c r="U17" s="4" t="inlineStr">
+        <is>
+          <t>DRN-3022853.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="120" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>EOW-017</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>DRN-3053156</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Aviva Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>18 Oct 2021</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Leaking asbestos pipe in garage of unoccupied estate property; Aviva initially mishandled claim, then agreed to replace pipe but applied £1,000 EOW excess; dispute over whether EOW excess was triggered when no water damage to property occurred</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>Leaking asbestos pipe in garage</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Unoccupied residential property</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Accepted — Disputed Settlement</t>
+        </is>
+      </c>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>Aviva applied £1,000 EOW excess endorsement asserting the claim was an escape of water claim; policyholder argued standard £175 excess applied as no water damage resulted from the pipe</t>
+        </is>
+      </c>
+      <c r="K18" s="3" t="inlineStr">
+        <is>
+          <t>Policyholder relied on policy schedule (standard excess £175) and photographs showing only a small puddle on the concrete garage floor that dried up and was not part of any repair; Aviva relied on the policy's EOW excess endorsement (£1,000 for damage caused by or resulting from EOW)</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M18" s="3" t="inlineStr">
+        <is>
+          <t>FOS required Aviva to reduce excess to £175 (no EOW damage occurred; claim was for specialist asbestos pipe removal and replacement, not water damage); required Aviva to pay £300 compensation for handling failures if not already paid</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P18" s="3" t="inlineStr">
+        <is>
+          <t>EOW excess endorsement (£1,000) applies only to 'damage caused by or resulting from Escape of Water from any Tank Apparatus or Pipe'; where the claim is for pipe replacement only and no such damage occurred, the standard excess applies; Trace and Access cover is only triggered where damage from EOW is present or reasonably anticipated</t>
+        </is>
+      </c>
+      <c r="Q18" s="3" t="inlineStr">
+        <is>
+          <t>Aviva's internal records of how the claim was categorised from the outset; full scope of agreed works under the settlement</t>
+        </is>
+      </c>
+      <c r="R18" s="3" t="inlineStr">
+        <is>
+          <t>No damage arose from escape of water — claim was for specialist removal of an asbestos pipe that trickled when water was switched on; the property was unoccupied and facilities unused; Aviva's own handling error led it to cover pipe replacement costs it was not obliged to cover; charging the higher EOW excess on top of that was unreasonable; Aviva gave conflicting excess amounts (£175, £250, £1,000) causing further confusion</t>
+        </is>
+      </c>
+      <c r="S18" s="3" t="inlineStr">
+        <is>
+          <t>EOW excess only triggers when property damage is caused by or results from escape of water; a claim for pipe removal or replacement without associated water damage attracts only the standard excess; insurers must communicate the basis for excess tier clearly and consistently</t>
+        </is>
+      </c>
+      <c r="T18" s="3" t="inlineStr">
+        <is>
+          <t>IF claim_type = pipe_removal_or_replacement AND no_water_damage_to_property THEN eow_excess = NOT applicable AND standard_excess APPLIES</t>
+        </is>
+      </c>
+      <c r="U18" s="2" t="inlineStr">
+        <is>
+          <t>DRN-3053156.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="120" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>EOW-018</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>DRN-3078337</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>QIC Europe Ltd</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>1 Nov 2021</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Burst mains stopcock pipe in ground floor bathroom; insurer repudiated trace and access claim on grounds the source was already visible and was outside the policy T&amp;A ambit</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>Mains stopcock pipe, ground floor bathroom</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I19" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>QIC argued T&amp;A cover did not apply because: (1) the mains stopcock was outside the policy T&amp;A ambit; (2) the leak source was already visible and did not need to be located; (3) no structural damage had actually occurred</t>
+        </is>
+      </c>
+      <c r="K19" s="5" t="inlineStr">
+        <is>
+          <t>Policyholder relied on plumber's invoice (£1,800 T&amp;A + £500 pipe repair) and 12 photographs; QIC relied on in-house surveying team's review and argued only cupboard removal was needed</t>
+        </is>
+      </c>
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M19" s="5" t="inlineStr">
+        <is>
+          <t>FOS directed QIC to pay T&amp;A costs of £1,800 less £750 policy excess, plus 8% simple interest from date Mr C paid invoice to date of settlement; pipe repair costs (£500) excluded as pipe repairs are excluded under policy terms</t>
+        </is>
+      </c>
+      <c r="N19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P19" s="5" t="inlineStr">
+        <is>
+          <t>T&amp;A cover applies to 'reasonable and necessary costs to remove any part of the building to find the source of the damage caused by water escaping from any fixed water or heating installation, apparatus or pipes'; T&amp;A applies even where the source location is approximately known but cannot be physically accessed; T&amp;A applies even where no damage has yet materialised if the policyholder acted reasonably to mitigate; pipe repair costs remain excluded even under a valid T&amp;A claim</t>
+        </is>
+      </c>
+      <c r="Q19" s="5" t="inlineStr">
+        <is>
+          <t>QIC did not appoint its own contractor to undertake T&amp;A; no independent assessment of what T&amp;A work would have cost from an approved contractor</t>
+        </is>
+      </c>
+      <c r="R19" s="5" t="inlineStr">
+        <is>
+          <t>It was unfair to decline T&amp;A because the location was known but not accessible — the specific pipe could not be confirmed until physically reached; if Mr C had not acted, significant damage would likely have resulted; QIC encouraged him to proceed but then repudiated; the T&amp;A invoice was proportionate given the extent of access work required (cupboard section, water softener pipes, waste pipe section, concrete floor); since QIC failed to appoint its own contractor, it cannot cap recovery to a lower hypothetical approved-contractor rate</t>
+        </is>
+      </c>
+      <c r="S19" s="5" t="inlineStr">
+        <is>
+          <t>T&amp;A cover is triggered when a leak exists and physical access to the source is obstructed, regardless of whether the approximate source location is known; insurers who fail to appoint their own T&amp;A contractor cannot subsequently restrict the policyholder's recovery to hypothetical approved contractor rates; pipe repair costs are excluded even within a valid T&amp;A claim</t>
+        </is>
+      </c>
+      <c r="T19" s="5" t="inlineStr">
+        <is>
+          <t>IF eow_confirmed AND leak_source_approximately_known AND physical_access_blocked THEN T&amp;A_cover = applicable; IF insurer_did_not_appoint_own_T&amp;A_contractor THEN insurer_cannot_reduce_recovery_to_approved_contractor_rate</t>
+        </is>
+      </c>
+      <c r="U19" s="4" t="inlineStr">
+        <is>
+          <t>DRN-3078337.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="120" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>EOW-019</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>DRN-3121008</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>AXA Insurance UK Plc</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>19 Nov 2021</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Leasehold flat; storage tank overflowed twice (16 months apart) from the same component (ball valve and overflow pipe); insurer registered second incident as a separate claim with a second excess; policyholder argued second incident resulted from the insurer's ineffective first repair</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>Storage tank overflow — faulty ball valve and overflow pipe (both incidents)</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Leasehold flat</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Accepted — Disputed Settlement</t>
+        </is>
+      </c>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>AXA asserted the second escape of water had a different cause to the first and should be treated as a new claim attracting a new excess of £1,500</t>
+        </is>
+      </c>
+      <c r="K20" s="3" t="inlineStr">
+        <is>
+          <t>AXA relied on its 2020 report claiming a different fault; policyholder noted AXA's 2019 and 2020 reports both reference ball valve and overflow pipe failure; FOS observed: same component failed both times; second incident was the first real test of the repair (Ms K had not been away for any extended period between incidents); gap of 16 months does not demonstrate an effective repair</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M20" s="3" t="inlineStr">
+        <is>
+          <t>AXA must: refund second policy excess of £1,500; remove record of second claim; reimburse cost of second carpet damaged in second incident; pay £250 compensation for inconvenience and upset caused as previously offered if not already paid; reimburse any previously agreed but unpaid works</t>
+        </is>
+      </c>
+      <c r="N20" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P20" s="3" t="inlineStr">
+        <is>
+          <t>Insurer that confirms a repair is complete and explicitly reassures the policyholder the same incident will not recur becomes responsible for damage if the same component subsequently fails; second incident should be treated as an extension of the first claim where on balance it results from an ineffective repair; gap between incidents does not demonstrate repair effectiveness if the system was never tested during that period</t>
+        </is>
+      </c>
+      <c r="Q20" s="3" t="inlineStr">
+        <is>
+          <t>No independent engineering report from AXA demonstrating the 2020 fault was technically distinct from and unrelated to the 2019 repair</t>
+        </is>
+      </c>
+      <c r="R20" s="3" t="inlineStr">
+        <is>
+          <t>Same component (ball valve and overflow) failed on both occasions; the second incident occurred the next time the system was actually tested (Ms K went away for the first time since the first repair); AXA explicitly reassured Ms K the problem was fixed and she would not have the same issue if she went away — this reassurance transferred responsibility for an ineffective repair to AXA; the 16-month gap cannot be treated as evidence of an effective and lasting repair</t>
+        </is>
+      </c>
+      <c r="S20" s="3" t="inlineStr">
+        <is>
+          <t>If an insurer confirms a repair is complete and explicitly reassures a policyholder the same event will not recur, the insurer becomes liable for the second incident if the same component fails again; the second incident should be assessed as an extension of the first claim unless the insurer demonstrates a technically distinct and unrelated cause</t>
+        </is>
+      </c>
+      <c r="T20" s="3" t="inlineStr">
+        <is>
+          <t>IF second_eow_incident AND same_component_failed AND insurer_confirmed_first_repair_complete AND policyholder_sought_explicit_reassurance THEN second_incident = extension_of_first_claim AND second_excess = NOT payable</t>
+        </is>
+      </c>
+      <c r="U20" s="2" t="inlineStr">
+        <is>
+          <t>DRN-3121008.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="120" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>EOW-020</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>DRN-3517894</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>AA Underwriting Insurance Company Limited</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>5 Aug 2022</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Two EOW incidents: original kitchen damage from internal soil stack leak (accepted); second incident — bathroom floor lifting from bath waste pipe — occurred while first claim repairs were being completed; insurer registered second as a new claim; policyholder argued second leak caused by pipe disturbance during first repair</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>First: internal soil stack (kitchen); Second: bath waste pipe (disturbed during first repair)</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I21" s="4" t="inlineStr">
+        <is>
+          <t>Accepted — Disputed Settlement</t>
+        </is>
+      </c>
+      <c r="J21" s="5" t="inlineStr">
+        <is>
+          <t>AA argued the second leak was from clean water (bath waste) and therefore unrelated to the soil stack claim; asserted the bath was not disturbed during the original repair works</t>
+        </is>
+      </c>
+      <c r="K21" s="5" t="inlineStr">
+        <is>
+          <t>Policyholder provided photographs showing toilet and bath share an interconnected pipework system leading to a single outlet pipe; scope of original works confirmed toilet pan, hand basin and vanity unit were removed and refitted; AA argued the soil stack repair was unlikely to displace bath waste pipework</t>
+        </is>
+      </c>
+      <c r="L21" s="4" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M21" s="5" t="inlineStr">
+        <is>
+          <t>FOS directed AA Underwriting to: remove record of second claim from all internal and external databases; pay costs to trace and repair bath waste pipe including excess paid under home emergency policy with 8% simple interest; pay repair costs for all EOW damage; pay £200 compensation within 28 days</t>
+        </is>
+      </c>
+      <c r="N21" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="O21" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P21" s="5" t="inlineStr">
+        <is>
+          <t>A second EOW incident occurring during or directly attributable to repair of the first claim should not be recorded as a separate claim; insurer cannot register a secondary leak as a new claim if it is more likely than not caused by disturbance from the repair works; no second excess is payable</t>
+        </is>
+      </c>
+      <c r="Q21" s="5" t="inlineStr">
+        <is>
+          <t>No independent plumbing expert report on whether removal and refitting of toilet and hand basin could have displaced the bath waste pipe</t>
+        </is>
+      </c>
+      <c r="R21" s="5" t="inlineStr">
+        <is>
+          <t>Pipework from toilet, bath and hand basin all interconnected and lead into one common pipe; the scope of works for the first claim included removal and refitting of the toilet and hand basin; on balance of probabilities, disturbing this interconnected pipework likely nudged the bath waste pipe out of place; the second leak was more likely than not attributable to the first repair</t>
+        </is>
+      </c>
+      <c r="S21" s="5" t="inlineStr">
+        <is>
+          <t>When a second EOW incident occurs during or shortly after repair of the first claim, assess whether the repair works disturbed connected pipework before registering a new claim; if pipework is interlinked and the repair scope included adjacent fittings, the second incident should be assessed as part of the first claim</t>
+        </is>
+      </c>
+      <c r="T21" s="5" t="inlineStr">
+        <is>
+          <t>IF second_eow_leak AND first_claim_repair_in_progress AND pipework_interconnected AND repair_scope_included_adjacent_fittings THEN second_leak = likely_attributable_to_first_repair AND new_claim_registration = NOT appropriate</t>
+        </is>
+      </c>
+      <c r="U21" s="4" t="inlineStr">
+        <is>
+          <t>DRN-3517894.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="120" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>EOW-021</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>DRN-3606995</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Ageas Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>1 Sep 2022</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Two separate bathroom EOW incidents (August 2019: bath waste pipe seal failure; February 2020: pop-up plug/waste mechanism failure); disputes over multiple excesses, scope and quantum of repairs, alternative accommodation period, electrical damage, and VAT withholding</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>Bath waste pipe seal failure (first, August 2019); pop-up plug/waste mechanism failure (second, February 2020) — both attributed to old age and wear</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Handling / Reinstatement Dispute</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>Ageas accepted both claims (£500 cash settlement for bathroom repairs) but refused to treat two EOW incidents as one claim; declined to extend alternative accommodation beyond 9 March 2020; declined electrical repair costs (no expert evidence linking to EOW); withheld VAT on cash settlement until proof of payment; settled only on scope identified by surveyor</t>
+        </is>
+      </c>
+      <c r="K22" s="3" t="inlineStr">
+        <is>
+          <t>Policyholder alleged structural instability, electrical damage, and extensive additional damage beyond surveyor's findings; Ageas relied on its own surveyor's May 2020 report (leaks localised and short-lived; no structural damage; electrics unrelated to EOW); policyholder's own loss adjuster friend agreed floor instability was from swelling laminate, not structural weakness</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M22" s="3" t="inlineStr">
+        <is>
+          <t>FOS confirmed Ageas did not need to do anything more; £200 compensation already paid by Ageas was sufficient; surveyor-based £500 settlement was fair; alternative accommodation covered only to 9 March 2020; two excesses correctly charged for two separate incidents with different physical causes; electrical repairs excluded (no expert evidence linking to EOW); VAT withholding until proof of payment is standard practice</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P22" s="3" t="inlineStr">
+        <is>
+          <t>Each separate EOW incident with a different physical cause attracts its own excess; policy covers repair to pre-loss condition only (like-for-like); VAT not payable on cash settlements until proof of payment to a VAT-registered contractor is provided; alternative accommodation ceases when insurer makes its position clear and property is not demonstrably uninhabitable</t>
+        </is>
+      </c>
+      <c r="Q22" s="3" t="inlineStr">
+        <is>
+          <t>Independent electrician's report linking electrical failure to EOW; itemised invoices separating EOW repair costs from wider renovation work; expert evidence linking floor instability to EOW rather than laminate swelling</t>
+        </is>
+      </c>
+      <c r="R22" s="3" t="inlineStr">
+        <is>
+          <t>Two incidents had genuinely different physical causes (seal failure vs pop-up mechanism failure); insurer's surveyor and policyholder's own loss adjuster friend agreed bathroom was not uninhabitable; no expert evidence linked electrical failure to EOW; insurer's expert evidence was strong and consistent at each decision point; £200 compensation was proportionate to communication failures</t>
+        </is>
+      </c>
+      <c r="S22" s="3" t="inlineStr">
+        <is>
+          <t>Two EOW incidents with different physical causes are separate claims attracting separate excesses; insurer's surveyor report is the primary basis for scoping repairs and assessing habitability; electrical damage requires expert evidence linking failure specifically to EOW; alternative accommodation liability ceases when insurer communicates clearly that the property is habitable and payments will stop</t>
+        </is>
+      </c>
+      <c r="T22" s="3" t="inlineStr">
+        <is>
+          <t>IF two_eow_incidents AND physically_different_causes THEN separate_claims AND separate_excesses = applicable; IF electrical_damage_claimed AND no_expert_report_linking_to_eow THEN electrical_claim = NOT covered</t>
+        </is>
+      </c>
+      <c r="U22" s="2" t="inlineStr">
+        <is>
+          <t>DRN-3606995.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="120" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>EOW-022</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>DRN-3860121</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Tesco Underwriting Limited</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>12 Jan 2023</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Three central heating pipe leaks in screed floor (kitchen, hallway, bathroom) discovered during major property renovation; insurer accepted claim but offered only £3,180.10, excluding items it considered renovation-related and reducing costs via unsupported surveyor annotations</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>Central heating pipes embedded in screed floor — kitchen, hallway and bathroom</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>Handling / Reinstatement Dispute</t>
+        </is>
+      </c>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t>Accepted — Disputed Settlement</t>
+        </is>
+      </c>
+      <c r="J23" s="5" t="inlineStr">
+        <is>
+          <t>Tesco argued many claimed items were renovation-related not EOW-related; applied surveyor's pencil cost annotations based on local knowledge without supporting market evidence; declined alternative accommodation invoice due to address error on invoice</t>
+        </is>
+      </c>
+      <c r="K23" s="5" t="inlineStr">
+        <is>
+          <t>Tesco relied on surveyor's unsubstantiated cost annotations; Mr C relied on original surveyor damage report, damage restoration specialist's moisture readings confirming affected rooms, itemised schedule of costs, and receipts/invoices; FOS found Tesco's annotations lacked market evidence</t>
+        </is>
+      </c>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M23" s="5" t="inlineStr">
+        <is>
+          <t>FOS directed Tesco to pay £11,600.29 total settlement (kitchen/hallway drying and rescreeding £1,533; bathroom/en-suite strip-out, tiling and reinstatement £3,403.61; bedroom joinery, flooring and redecoration £4,765.68; skip hire £348; T&amp;A investigative work £350; alternative accommodation £1,200) less any sum already paid, plus 8% statutory interest</t>
+        </is>
+      </c>
+      <c r="N23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O23" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P23" s="5" t="inlineStr">
+        <is>
+          <t>Insurer must handle claims promptly and fairly; surveyor cost reductions require supporting market evidence to be persuasive; only rooms identified in contemporaneous professional reports as EOW-affected are eligible for settlement; investigative work (T&amp;A) is covered; alternative accommodation is covered for the period the property is genuinely uninhabitable due to EOW repairs</t>
+        </is>
+      </c>
+      <c r="Q23" s="5" t="inlineStr">
+        <is>
+          <t>Itemised invoices clearly separating EOW repair costs from renovation costs; building schedule and control documents requested by Tesco but not provided; market cost evidence to support Tesco's reduced settlement figures</t>
+        </is>
+      </c>
+      <c r="R23" s="5" t="inlineStr">
+        <is>
+          <t>Tesco's 4-month delay in accepting the claim was unjustified — surveyor's report was available by end of November; Mr C's decision to proceed with repairs during the delay was reasonable given ongoing renovation and builders already on site; surveyor's pencil annotations without documentary support were not persuasive — insurer must evidence that materials and labour could be sourced at the annotated rates; coverage limited to rooms identified in contemporaneous damage assessment reports</t>
+        </is>
+      </c>
+      <c r="S23" s="5" t="inlineStr">
+        <is>
+          <t>A prolonged delay in accepting a claim forces the policyholder to proceed without authorisation; FOS will hold the insurer responsible for reasonable repair costs incurred during that delay; surveyor cost reductions must be evidenced by market data, not bare assertions; rooms not identified in the contemporaneous damage report are excluded even if costs were incurred there</t>
+        </is>
+      </c>
+      <c r="T23" s="5" t="inlineStr">
+        <is>
+          <t>IF claim_acceptance_delay &gt; 60_days AND policyholder_proceeds_with_repairs THEN insurer_cannot_reject_reasonable_costs_incurred_during_delay; IF surveyor_cost_reduction AND no_market_evidence_provided THEN cost_reduction = NOT accepted</t>
+        </is>
+      </c>
+      <c r="U23" s="4" t="inlineStr">
+        <is>
+          <t>DRN-3860121.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="120" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>EOW-023</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>DRN-4205492</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>QIC Europe Limited</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>8 Sep 2023</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>Two EOW incidents: first was bathroom leak damaging kitchen (accepted and repaired by QIC's contractor); second was a kitchen leak from the area QIC's contractor had been working on, a few weeks after first repair; insurer argued second was an independent frozen pipe event and opened a new claim</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>First: bathroom pipe; Second: isolator valve in kitchen fitted by QIC's contractor (cracked weeks after installation)</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>Accepted — Disputed Settlement</t>
+        </is>
+      </c>
+      <c r="J24" s="3" t="inlineStr">
+        <is>
+          <t>QIC argued the second leak was caused by water freezing in the pipe (outside temperature -3.6°C on the day) and was therefore an independent event warranting a separate claim and separate excess</t>
+        </is>
+      </c>
+      <c r="K24" s="3" t="inlineStr">
+        <is>
+          <t>QIC provided outside weather data (-3.6°C) and an industry article on frozen pipe claims; policyholder argued QIC's contractor's valve was defective or incorrectly fitted; FOS noted outside temperature is not the same as enclosed indoor pipe temperature; the freeze-claims article QIC cited referred to dates 10 days after Mr A's claim</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M24" s="3" t="inlineStr">
+        <is>
+          <t>FOS directed QIC to: treat both leaks as one claim including kitchen floor tiles; charge only one excess and refund second if already paid; pay £150 compensation for service shortfalls and avoidable delays</t>
+        </is>
+      </c>
+      <c r="N24" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P24" s="3" t="inlineStr">
+        <is>
+          <t>A second leak originating from an area where the insurer's contractor recently worked is prima facie attributable to the contractor's work unless the insurer establishes an independent cause; a valve cracking within weeks of installation suggests manufacturing defect or incorrect fitting; insurer is responsible for its appointed contractor's workmanship</t>
+        </is>
+      </c>
+      <c r="Q24" s="3" t="inlineStr">
+        <is>
+          <t>Engineering inspection of the cracked valve to determine whether failure was from freeze damage or installation defect; indoor temperature data for the property on the day of the leak</t>
+        </is>
+      </c>
+      <c r="R24" s="3" t="inlineStr">
+        <is>
+          <t>Valve cracked within weeks of installation in the specific area QIC's contractor had worked on; outside temperature of -3.6°C does not establish that an enclosed kitchen cupboard pipe was at freezing temperatures; freeze-claim surge article cited by QIC referred to a later date; on balance, valve more likely failed due to defect or improper installation; QIC is responsible for its contractor's work</t>
+        </is>
+      </c>
+      <c r="S24" s="3" t="inlineStr">
+        <is>
+          <t>When a second EOW incident occurs in the area recently worked on by the insurer's contractor, the presumption is the contractor caused it; insurer cannot rebut this by citing weather data alone without establishing indoor pipe temperatures; insurer is liable for its contractor's workmanship failures</t>
+        </is>
+      </c>
+      <c r="T24" s="3" t="inlineStr">
+        <is>
+          <t>IF second_leak_location = area_of_recent_insurer_contractor_work AND time_since_repair &lt; 60_days THEN second_leak = presumptively_attributable_to_contractor AND separate_claim = NOT appropriate UNLESS independent_cause_established</t>
+        </is>
+      </c>
+      <c r="U24" s="2" t="inlineStr">
+        <is>
+          <t>DRN-4205492.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="120" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>EOW-024</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>DRN-4223988</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>HDI Global Speciality SE</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>8 Jan 2024</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>Residential EOW claim for damage from leaking 15mm water supply pipe under floor of rear extension (2019); insurer declined after initial inspection found no evidence of leak; policyholder later produced builder's report confirming pipe found and capped, and water bills showing anomalous usage during the claim period</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>15mm water supply pipe under floor in rear extension</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I25" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J25" s="5" t="inlineStr">
+        <is>
+          <t>HDI's inspection (June 2019) found no evidence of an escape of water; water mains sound test found no water supply leaks; HDI questioned why the builder's report was not shared until long after the 2019 inspection</t>
+        </is>
+      </c>
+      <c r="K25" s="5" t="inlineStr">
+        <is>
+          <t>HDI relied on June 2019 inspection report (no leak found) and water mains sound test; policyholder provided: (1) builder's statement (November 2019) with photographs confirming leaking pipe found and capped, bathroom left inoperable; (2) water bills showing usage spike from ~15-19m3 per period to 63m3 in Feb-Aug 2019, reducing back to normal after pipe was capped in November 2019</t>
+        </is>
+      </c>
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M25" s="5" t="inlineStr">
+        <is>
+          <t>FOS directed HDI to pay Ms L £600 compensation for handling failures; HDI must reconsider the EOW claim based on new evidence; if the claim proceeds to settlement, HDI must settle subject to remaining policy terms and limits (note: this direction does not affect the separate declined subsidence claim)</t>
+        </is>
+      </c>
+      <c r="N25" s="4" t="n">
+        <v>600</v>
+      </c>
+      <c r="O25" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P25" s="5" t="inlineStr">
+        <is>
+          <t>Insurer must investigate EOW claims thoroughly; where an initial inspection is inconclusive and leaves open the possibility of an undetected leak, the insurer should not issue a final decline without pursuing further investigation; subsequently produced evidence (builder's report, utility bills) must be properly evaluated before a final position is maintained</t>
+        </is>
+      </c>
+      <c r="Q25" s="5" t="inlineStr">
+        <is>
+          <t>Builder's report and water bills were not provided to HDI until after the initial inspection; no independent assessment of whether damp damage was caused by EOW vs subsidence or rising damp (separate subsidence claim exists)</t>
+        </is>
+      </c>
+      <c r="R25" s="5" t="inlineStr">
+        <is>
+          <t>Water bills showing usage rising from ~15-19m3 per period to 63m3 during the claimed EOW period, then reducing to normal after the pipe was capped, constitutes strong circumstantial evidence of an ongoing underground leak; builder's report confirms leaking pipe was found and capped; HDI's own inspection acknowledged a remote possibility of an undetected pipe leak; on balance, sufficient evidence that an EOW did take place; £600 compensation is proportionate to HDI's handling failures over several years</t>
+        </is>
+      </c>
+      <c r="S25" s="5" t="inlineStr">
+        <is>
+          <t>Water utility bill anomalies — a significant usage spike coinciding with the claimed EOW period, returning to normal after the source is capped — are strong circumstantial evidence of a leak even where an initial physical inspection found no visible damage; insurers should consider requesting utility bills as standard evidence in EOW investigations, especially where underground or concealed pipework is involved</t>
+        </is>
+      </c>
+      <c r="T25" s="5" t="inlineStr">
+        <is>
+          <t>IF initial_inspection_inconclusive AND water_bills_show_usage_spike_during_claim_period AND usage_returns_to_normal_after_capping THEN EOW = likely_occurred AND full_decline = NOT defensible</t>
+        </is>
+      </c>
+      <c r="U25" s="4" t="inlineStr">
+        <is>
+          <t>DRN-4223988.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="120" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>EOW-025</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>DRN-4227214</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Saga Services Limited</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>11 Oct 2023</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>Unoccupied residential property; leak occurred and claim made; insurer declined under endorsement limiting cover to FLEA only (fire, smoke, lightning, aircraft impact); complainants alleged mis-selling and that the EOW exclusion was not made clear during the sales call</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>Not specified (property had a leak)</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Unoccupied residential property</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>Policy contained an endorsement restricting cover to FLEA only, explicitly excluding EOW for properties unoccupied for more than 60 consecutive days; endorsement was in place and disclosed at point of sale</t>
+        </is>
+      </c>
+      <c r="K26" s="3" t="inlineStr">
+        <is>
+          <t>Complainants alleged sales agent verbally confirmed EOW cover during the call; Saga relied on sales call recordings showing agent stated FLEA-only cover at least twice and read the endorsement in full; IPID stated EOW excluded for properties unoccupied 60+ consecutive days; no recording evidence that EOW was confirmed as covered</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M26" s="3" t="inlineStr">
+        <is>
+          <t>FOS did not uphold; Saga adequately disclosed the FLEA-only endorsement during the sales call and in policy documents including the IPID; £250 compensation already paid by Saga for administrative errors was sufficient; FOS could not reasonably ask Saga to do anything more</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P26" s="3" t="inlineStr">
+        <is>
+          <t>Unoccupied property endorsement restricting cover to FLEA only (excluding EOW) is a standard and not unusual market practice; insurer adequately discharges its disclosure obligation by reading the endorsement in full during the sales call and providing a clear IPID stating the exclusion; a non-advised sale places the onus on the policyholder to verify the policy meets their needs</t>
+        </is>
+      </c>
+      <c r="Q26" s="3" t="inlineStr">
+        <is>
+          <t>No recording evidence that the sales agent verbally confirmed EOW cover (FOS reviewed recordings — no such statement found); complainants produced no evidence they queried EOW cover during the call</t>
+        </is>
+      </c>
+      <c r="R26" s="3" t="inlineStr">
+        <is>
+          <t>Sales call recordings confirmed agent stated FLEA-only cover at least twice and read the endorsement in full; IPID clearly stated EOW excluded for properties unoccupied 60+ consecutive days; endorsement is standard and not unusual for unoccupied properties; as a non-advised sale, onus was on complainants to ensure the policy met their needs; at no point during the call did the agent state EOW was covered</t>
+        </is>
+      </c>
+      <c r="S26" s="3" t="inlineStr">
+        <is>
+          <t>Where an unoccupied property endorsement excludes EOW and the insurer can demonstrate the endorsement was clearly disclosed during the sales call and in policy documents, the decline is defensible; FOS will not uphold mis-selling claims where the insurer's sales records demonstrate adequate, unambiguous disclosure</t>
+        </is>
+      </c>
+      <c r="T26" s="3" t="inlineStr">
+        <is>
+          <t>IF policy_type = unoccupied AND endorsement_excludes_eow AND insurer_read_endorsement_during_sales_call AND IPID_states_eow_excluded THEN mis_selling_claim = NOT upheld AND coverage_decline = defensible</t>
+        </is>
+      </c>
+      <c r="U26" s="2" t="inlineStr">
+        <is>
+          <t>DRN-4227214.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add EOW-036 to EOW-057 to Escape of Water Case Database
Appends the final 22 FOS decision cases (EOW-036 through EOW-057) to
Escape_of_Water_Case_Database.xlsx, bringing the total to 57 cases and
completing processing of all available EOW PDFs.

Updates PROJECT_STATUS.md to reflect completion and clears the next-batch
section. Updates append_eow_v2.py with the new case data.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/knowledge/case-databases/Escape_of_Water_Case_Database.xlsx
+++ b/knowledge/case-databases/Escape_of_Water_Case_Database.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U36"/>
+  <dimension ref="A1:U58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4278,6 +4278,2300 @@
         </is>
       </c>
     </row>
+    <row r="37" ht="120" customHeight="1">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>EOW-036</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>DRN-5088221</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>Accelerant Insurance Europe SA/NV UK Branch</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>15 Nov 2024</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>Escape of water causing ceiling damage in a social housing property; insurer declined citing prior workmanship as cause rather than EOW; £200 compensation directed for unexplained 3-month handling delay only</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="inlineStr">
+        <is>
+          <t>Disputed — surveyor attributed ceiling cracking to prior defective workmanship rather than EOW; freeholder unable to confirm a water event occurred</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>Residential home (rented to local council — social housing)</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I37" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J37" s="5" t="inlineStr">
+        <is>
+          <t>Surveyor attributed ceiling cracking to prior defective workmanship; freeholder could not confirm an EOW event had occurred; insurer declined on causation grounds</t>
+        </is>
+      </c>
+      <c r="K37" s="5" t="inlineStr">
+        <is>
+          <t>Surveyor's report attributed ceiling damage to prior workmanship; freeholder's inability to confirm EOW event; 3-month unexplained handling delay not disputed</t>
+        </is>
+      </c>
+      <c r="L37" s="4" t="inlineStr">
+        <is>
+          <t>Upheld in Part</t>
+        </is>
+      </c>
+      <c r="M37" s="5" t="inlineStr">
+        <is>
+          <t>FOS upheld only in relation to a 3-month unexplained handling delay; directed Accelerant to pay £200 compensation for that delay; coverage decline upheld</t>
+        </is>
+      </c>
+      <c r="N37" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="O37" s="4" t="inlineStr">
+        <is>
+          <t>No — Commercial</t>
+        </is>
+      </c>
+      <c r="P37" s="5" t="inlineStr">
+        <is>
+          <t>Where a surveyor attributes damage to prior workmanship rather than an escape of water, and the freeholder cannot confirm the water event, the insurer is entitled to decline on causation grounds; compensation remains available for unexplained handling delays even where coverage is not established</t>
+        </is>
+      </c>
+      <c r="Q37" s="5" t="inlineStr">
+        <is>
+          <t>Confirmation from the freeholder or maintenance records of an EOW event occurring at the property; independent assessment of whether ceiling cracking pattern was consistent with EOW or prior workmanship</t>
+        </is>
+      </c>
+      <c r="R37" s="5" t="inlineStr">
+        <is>
+          <t>Surveyor found no evidence linking ceiling cracking to an EOW event; freeholder's inability to confirm the event further weakened the causation claim; however, a 3-month unexplained handling delay warranted £200 compensation</t>
+        </is>
+      </c>
+      <c r="S37" s="5" t="inlineStr">
+        <is>
+          <t>Where a surveyor attributes damage to prior workmanship and the freeholder cannot confirm an EOW event, the coverage decline is sustainable; always investigate and compensate for unexplained handling delays even where the coverage decision is upheld</t>
+        </is>
+      </c>
+      <c r="T37" s="5" t="inlineStr">
+        <is>
+          <t>IF surveyor_attributes_damage_to_workmanship AND freeholder_cannot_confirm_eow THEN coverage_decline = defensible; IF unexplained_handling_delay_3_months_plus THEN compensation = payable_regardless_of_coverage_outcome</t>
+        </is>
+      </c>
+      <c r="U37" s="4" t="inlineStr">
+        <is>
+          <t>DRN-5088221.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="120" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>EOW-037</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>DRN-5193042</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Allied World Assurance Company (Europe) dac</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>21 Jan 2025</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>Escape of water from failed grouting and sealant around bath and shower at a tenanted property; insurer declined under gradually operating cause; £200 compensation directed for handling delay on a separate plasterwork element</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>Failed grouting and sealant around bath and shower enclosure — gradual deterioration over approximately 3 months</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>Residential home (tenanted landlord policy)</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J38" s="3" t="inlineStr">
+        <is>
+          <t>Failed grouting and sealant establishes gradual deterioration over approximately 3 months with landlord and tenant awareness; gradually operating cause exclusion properly applied</t>
+        </is>
+      </c>
+      <c r="K38" s="3" t="inlineStr">
+        <is>
+          <t>Insurer's inspection identified failed grouting and sealant with evidence of ongoing moisture damage over months; tenant and landlord were or ought to have been aware of the deteriorating condition; £200 compensation directed for a separate handling delay on the plasterwork element</t>
+        </is>
+      </c>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M38" s="3" t="inlineStr">
+        <is>
+          <t>FOS did not uphold the EOW coverage dispute — gradually operating cause exclusion properly applied; directed Allied World to pay £200 compensation for a handling delay on a separate plasterwork element</t>
+        </is>
+      </c>
+      <c r="N38" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="O38" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P38" s="3" t="inlineStr">
+        <is>
+          <t>Failed grouting and sealant around bathroom fixtures establishes a gradually operating cause; where damage has been occurring over approximately 3 months and the landlord and tenant were or ought to have been aware, the gradual cause exclusion is properly applied; compensation is available for handling failures on separate claim elements even where the main coverage decision is upheld</t>
+        </is>
+      </c>
+      <c r="Q38" s="3" t="inlineStr">
+        <is>
+          <t>Independent assessment of precisely when the grouting failure began and whether it was reasonably discoverable by the tenant or landlord; evidence of the landlord's inspection schedule and whether the property was checked during the deterioration period</t>
+        </is>
+      </c>
+      <c r="R38" s="3" t="inlineStr">
+        <is>
+          <t>Failed grouting and sealant is a classic gradual deterioration scenario; approximately 3 months of deterioration with parties who were or ought to have been aware means the exclusion applies; handling delay on the plasterwork element warranted £200 compensation</t>
+        </is>
+      </c>
+      <c r="S38" s="3" t="inlineStr">
+        <is>
+          <t>Failed grouting and sealant damage should always be assessed against the gradual cause exclusion — the duration of deterioration and whether the policyholder or tenant was aware are the key questions; compensation may still be awarded for handling failures even where the coverage decision is upheld</t>
+        </is>
+      </c>
+      <c r="T38" s="3" t="inlineStr">
+        <is>
+          <t>IF eow_source_is_failed_grouting_or_sealant AND deterioration_duration_3_months_plus AND landlord_or_tenant_ought_to_have_known THEN gradual_cause_exclusion = applicable; IF handling_delay_on_separate_claim_element THEN compensation_available_regardless_of_coverage_decision</t>
+        </is>
+      </c>
+      <c r="U38" s="2" t="inlineStr">
+        <is>
+          <t>DRN-5193042.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="120" customHeight="1">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>EOW-038</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>DRN-5198749</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>Accredited Insurance (Europe) Ltd</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>4 Feb 2025</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>Burst pipe caused by freezing discovered after policyholder switched insurers; dispute over which insurer's policy period covers the loss</t>
+        </is>
+      </c>
+      <c r="F39" s="5" t="inlineStr">
+        <is>
+          <t>Burst pipe — frozen pipe failure; exact date of burst disputed between prior insurer (Accredited) and new insurer</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H39" s="4" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I39" s="4" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="J39" s="5" t="inlineStr">
+        <is>
+          <t>Dispute was between insurers about which policy period the loss fell within — Accredited (on risk during the likely freeze period) sought to decline; new insurer argued the damage occurred after their coverage began</t>
+        </is>
+      </c>
+      <c r="K39" s="5" t="inlineStr">
+        <is>
+          <t>Weather data showing sub-zero temperatures during Accredited's policy period; electricity tripping as corroborating evidence of the likely freeze event timing; Accredited's weather data analysis vs new insurer's position on discovery date</t>
+        </is>
+      </c>
+      <c r="L39" s="4" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M39" s="5" t="inlineStr">
+        <is>
+          <t>FOS upheld — Accredited Insurance (Europe) Ltd to accept the claim as the insurer on risk during the likely freeze period; directed to pay £500 compensation for distress and inconvenience; may seek contribution from the successor insurer</t>
+        </is>
+      </c>
+      <c r="N39" s="4" t="n">
+        <v>500</v>
+      </c>
+      <c r="O39" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P39" s="5" t="inlineStr">
+        <is>
+          <t>The relevant date for a frozen pipe loss is the date of the freeze event, not the date of discovery; weather data (sub-zero temperatures) and corroborating physical evidence (electricity tripping) are sufficient to establish which policy period a frozen pipe loss falls within; the insurer on risk during the likely freeze period takes the lead and can seek contribution from the successor insurer</t>
+        </is>
+      </c>
+      <c r="Q39" s="5" t="inlineStr">
+        <is>
+          <t>Precise date the pipe burst confirmed by independent expert; specific temperature readings at the property location on the relevant dates</t>
+        </is>
+      </c>
+      <c r="R39" s="5" t="inlineStr">
+        <is>
+          <t>Weather data established sub-zero temperatures during Accredited's policy period; electricity tripping corroborated the timing of the freeze event; date of discovery is not determinative for a freeze-pipe loss — the relevant date is when conditions causing the burst occurred; Accredited was on risk at that time</t>
+        </is>
+      </c>
+      <c r="S39" s="5" t="inlineStr">
+        <is>
+          <t>For frozen pipe losses, always establish the likely date of the freeze event using weather data and corroborating evidence (electricity trips, witness accounts), not just the date of discovery; the insurer on risk at the time of the freeze event bears primary liability regardless of when the damage became visible</t>
+        </is>
+      </c>
+      <c r="T39" s="5" t="inlineStr">
+        <is>
+          <t>IF frozen_pipe_loss AND weather_data_shows_sub_zero_during_prior_insurer_period AND corroborating_evidence_supports_freeze_timing THEN prior_insurer = liable; IF policyholder_switches_insurer AND loss_date_disputed THEN use_freeze_event_date_not_discovery_date</t>
+        </is>
+      </c>
+      <c r="U39" s="4" t="inlineStr">
+        <is>
+          <t>DRN-5198749.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="120" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>EOW-039</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>DRN-5199107</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Admiral Insurance (Gibraltar) Limited</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>11 Feb 2025</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>Accepted EOW claim at a property being marketed for sale; dispute about occupancy enquiries, market value reduction, and adequacy of cash settlement</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>Not specified — EOW claim accepted by Admiral; dispute concerns handling and settlement, not the EOW source</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Residential home (being marketed for sale at time of claim)</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>Handling / Reinstatement Dispute</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="J40" s="3" t="inlineStr">
+        <is>
+          <t>N/A — claim accepted; Admiral disputed certain elements of the extended settlement process including additional losses alleged to result from property being sold at auction under financial pressure</t>
+        </is>
+      </c>
+      <c r="K40" s="3" t="inlineStr">
+        <is>
+          <t>Policyholder alleged Admiral's occupancy enquiries caused delay leading to forced auction sale at undervalue; Admiral's extended enquiries based on minimal furniture and property being marketed for sale; FOS found occupancy enquiries reasonable; market value reduction from repair not a covered loss; £525 D&amp;I compensation paid by Admiral confirmed as fair</t>
+        </is>
+      </c>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M40" s="3" t="inlineStr">
+        <is>
+          <t>FOS did not uphold — Admiral's occupancy enquiries were reasonable; insurer not responsible for policyholder's decision to sell at auction; market value reduction from repair not a covered loss; cash settlement (£43,243 plus interest) confirmed as correct; Admiral's existing £525 compensation payment confirmed as adequate</t>
+        </is>
+      </c>
+      <c r="N40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O40" s="2" t="inlineStr">
+        <is>
+          <t>No — Handling Dispute</t>
+        </is>
+      </c>
+      <c r="P40" s="3" t="inlineStr">
+        <is>
+          <t>Where a property shows minimal furniture and is being marketed for sale, an insurer is entitled to make extended occupancy enquiries before progressing an EOW claim; market value reduction resulting from disclosed repair history is not a consequential loss covered under the policy; an insurer is not responsible for a policyholder's voluntary decision to sell at auction under financial pressure</t>
+        </is>
+      </c>
+      <c r="Q40" s="3" t="inlineStr">
+        <is>
+          <t>Evidence linking Admiral's handling delay directly to the decision to sell at auction; independent valuation confirming the market value reduction specifically attributable to the EOW repair work</t>
+        </is>
+      </c>
+      <c r="R40" s="3" t="inlineStr">
+        <is>
+          <t>Admiral's enquiries were reasonable given the property was sparsely furnished and being marketed for sale; the decision to sell at auction under financial pressure was the policyholder's own; market value reduction from disclosed repair history is consequential loss and not covered; £525 compensation already paid by Admiral was fair for any handling inconvenience</t>
+        </is>
+      </c>
+      <c r="S40" s="3" t="inlineStr">
+        <is>
+          <t>Extended occupancy enquiries are justified where a property is minimally furnished and being marketed for sale; the insurer is not responsible for consequential financial decisions the policyholder makes during the claims process; always confirm whether D&amp;I compensation has already been paid before making an additional award</t>
+        </is>
+      </c>
+      <c r="T40" s="3" t="inlineStr">
+        <is>
+          <t>IF property_minimally_furnished AND being_marketed_for_sale THEN occupancy_enquiries = justified; IF market_value_reduction_from_repair_history THEN consequential_loss = NOT covered; IF insurer_already_paid_di_compensation AND fos_confirms_adequate THEN no_additional_award</t>
+        </is>
+      </c>
+      <c r="U40" s="2" t="inlineStr">
+        <is>
+          <t>DRN-5199107.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="120" customHeight="1">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>EOW-040</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>DRN-5396824</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>Aviva Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>16 Apr 2025</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>Escape of water from under-floor waste pipe; claim accepted but dispute about whether kitchen unit damage was caused by the EOW and whether compensation for poor expectation management was adequate</t>
+        </is>
+      </c>
+      <c r="F41" s="5" t="inlineStr">
+        <is>
+          <t>Under-floor waste pipe (kitchen area)</t>
+        </is>
+      </c>
+      <c r="G41" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H41" s="4" t="inlineStr">
+        <is>
+          <t>Handling / Reinstatement Dispute</t>
+        </is>
+      </c>
+      <c r="I41" s="4" t="inlineStr">
+        <is>
+          <t>Accepted — Disputed Settlement</t>
+        </is>
+      </c>
+      <c r="J41" s="5" t="inlineStr">
+        <is>
+          <t>Aviva declined to include kitchen unit damage in scope — expert evidence showed wastewater from the under-floor waste pipe did not reach joist height; kitchen units not demonstrably damaged by the EOW</t>
+        </is>
+      </c>
+      <c r="K41" s="5" t="inlineStr">
+        <is>
+          <t>Policyholder argued kitchen units were damaged by the EOW; Aviva's expert evidence showed wastewater was confined to the floor void and did not reach joist height, meaning kitchen units were not in the flood path; inconsistent expert reports did not establish the link between kitchen unit damage and this specific EOW</t>
+        </is>
+      </c>
+      <c r="L41" s="4" t="inlineStr">
+        <is>
+          <t>Upheld in Part</t>
+        </is>
+      </c>
+      <c r="M41" s="5" t="inlineStr">
+        <is>
+          <t>FOS upheld in part — Aviva directed to increase compensation from £200 to £500 for poor expectation management during the claims process; kitchen unit coverage dispute not upheld — policyholder failed to establish the link between kitchen unit damage and this specific EOW event</t>
+        </is>
+      </c>
+      <c r="N41" s="4" t="n">
+        <v>500</v>
+      </c>
+      <c r="O41" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P41" s="5" t="inlineStr">
+        <is>
+          <t>Policyholder bears the burden of linking each claimed item to the specific EOW event; where expert evidence shows the escape was localised to the floor void and did not reach the height of kitchen units, there is no evidential basis for including unit damage in the scope; an insurer may be required to pay increased compensation for poor expectation management even where the coverage decision is upheld</t>
+        </is>
+      </c>
+      <c r="Q41" s="5" t="inlineStr">
+        <is>
+          <t>Independent expert evidence establishing that wastewater from the under-floor waste pipe reached the height of kitchen base units; photographic evidence of unit damage consistent with waterline from a floor void leak</t>
+        </is>
+      </c>
+      <c r="R41" s="5" t="inlineStr">
+        <is>
+          <t>Expert evidence showed wastewater confined to floor void below joist level — kitchen units not in the water path; inconsistent expert reports did not resolve the causation question in the policyholder's favour; however, Aviva's poor expectation management during the claim was separately established and warranted increased compensation from £200 to £500</t>
+        </is>
+      </c>
+      <c r="S41" s="5" t="inlineStr">
+        <is>
+          <t>Always obtain expert confirmation of the water path and maximum flood level before including items in a scope of works; poor expectation management during a claim can attract compensation even where the underlying coverage decision is correct; kitchen unit damage from a floor void pipe requires specific evidence the water reached unit level</t>
+        </is>
+      </c>
+      <c r="T41" s="5" t="inlineStr">
+        <is>
+          <t>IF eow_from_floor_void AND expert_confirms_water_did_not_reach_unit_level THEN unit_damage = NOT established; IF poor_expectation_management_during_claim THEN compensation = payable_even_if_coverage_decision_upheld</t>
+        </is>
+      </c>
+      <c r="U41" s="4" t="inlineStr">
+        <is>
+          <t>DRN-5396824.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="120" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>EOW-041</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>DRN5611706</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>CIS General Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr"/>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>Escape of water while property was unoccupied; insurer declined under EOW-when-unoccupied exclusion; adviser had explained the theft exclusion but not the separate EOW unoccupied exclusion</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>Escape of water during unoccupied period (specific source not detailed in this older decision)</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>Residential home (unoccupied at time of loss)</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J42" s="3" t="inlineStr">
+        <is>
+          <t>CIS declined under the EOW-when-unoccupied exclusion; policy defined unoccupied as insufficiently furnished for full habitation OR not lived in for 60 or more consecutive days — dual test</t>
+        </is>
+      </c>
+      <c r="K42" s="3" t="inlineStr">
+        <is>
+          <t>Policyholder stated the property was fully furnished; CIS's adviser at inception had explained the theft exclusion for unoccupied properties but had not explained the separate EOW exclusion; FOS found the failure to explain the EOW exclusion meant CIS could not properly rely on it</t>
+        </is>
+      </c>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M42" s="3" t="inlineStr">
+        <is>
+          <t>FOS upheld — CIS General Insurance Limited directed to accept and settle the claim; £200 compensation for distress and inconvenience; CIS must confirm whether the property met the unoccupied definition before relying on the exclusion</t>
+        </is>
+      </c>
+      <c r="N42" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="O42" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P42" s="3" t="inlineStr">
+        <is>
+          <t>Where an insurer's adviser explains one exclusion (theft when unoccupied) but not another (EOW when unoccupied), the insurer cannot subsequently rely on the unexplained exclusion; where a policyholder states the property was fully furnished, the insurer must also confirm the property satisfied the unoccupied definition (dual test: insufficiently furnished for full habitation OR not lived in for 60+ consecutive days) before invoking the exclusion</t>
+        </is>
+      </c>
+      <c r="Q42" s="3" t="inlineStr">
+        <is>
+          <t>Precise details of what the CIS adviser explained at inception; independent confirmation of the property's furnishing status at the time of the EOW; evidence of whether the 60-day non-habitation limb of the unoccupied definition was met</t>
+        </is>
+      </c>
+      <c r="R42" s="3" t="inlineStr">
+        <is>
+          <t>CIS's adviser explained the theft exclusion for unoccupied properties but failed to draw attention to the separate EOW exclusion; this failure means CIS cannot fairly rely on the EOW exclusion; additionally, the unoccupied definition involves a dual test and CIS had not confirmed both limbs were met given the policyholder's claim to be fully furnished</t>
+        </is>
+      </c>
+      <c r="S42" s="3" t="inlineStr">
+        <is>
+          <t>When explaining policy exclusions at inception or renewal, all relevant exclusions — not just some — must be drawn to the policyholder's attention; where an exclusion has a dual test (insufficiently furnished OR not lived in for 60+ days), both limbs must be assessed before the exclusion is invoked; failure to explain an exclusion prevents reliance on it</t>
+        </is>
+      </c>
+      <c r="T42" s="3" t="inlineStr">
+        <is>
+          <t>IF adviser_explained_one_unoccupied_exclusion AND did_not_explain_eow_unoccupied_exclusion THEN eow_unoccupied_exclusion = cannot_be_relied_upon; IF unoccupied_definition_is_dual_test AND policyholder_claims_furnished THEN both_limbs_must_be_assessed_before_exclusion_invoked</t>
+        </is>
+      </c>
+      <c r="U42" s="2" t="inlineStr">
+        <is>
+          <t>DRN5611706.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="120" customHeight="1">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>EOW-042</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>DRN-5649220</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>Aviva Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>16 Dec 2025</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>Escape of water at a tenanted rental property — kitchen floor damage accepted; dispute about whether wall and ceiling damage beyond the kitchen floor was also caused by the same EOW</t>
+        </is>
+      </c>
+      <c r="F43" s="5" t="inlineStr">
+        <is>
+          <t>Escape of water causing kitchen floor damage (source of broader wall and ceiling damage disputed)</t>
+        </is>
+      </c>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
+          <t>Residential home (tenanted rental property)</t>
+        </is>
+      </c>
+      <c r="H43" s="4" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I43" s="4" t="inlineStr">
+        <is>
+          <t>Accepted — Disputed Settlement</t>
+        </is>
+      </c>
+      <c r="J43" s="5" t="inlineStr">
+        <is>
+          <t>Aviva accepted kitchen floor damage but declined to extend coverage to walls and ceilings; damp specialist report was internally inconsistent — body cited a persistent water leak as cause but the associated quote described penetrating damp remediation; salt contamination in walls indicated external water ingress rather than internal EOW</t>
+        </is>
+      </c>
+      <c r="K43" s="5" t="inlineStr">
+        <is>
+          <t>Policyholder's damp specialist report attributed damage in body text to a persistent leak but provided a quote for penetrating damp remediation; salt contamination in walls was consistent with external water ingress, not EOW; FOS found the report's internal inconsistency and the salt contamination evidence undermined the claim that wall damage was caused by the EOW</t>
+        </is>
+      </c>
+      <c r="L43" s="4" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M43" s="5" t="inlineStr">
+        <is>
+          <t>FOS did not uphold — Aviva's decision to limit coverage to the confirmed kitchen floor area was fair; the damp specialist report's internal inconsistency and salt contamination evidence meant wall damage could not be reliably attributed to the EOW; no further award directed</t>
+        </is>
+      </c>
+      <c r="N43" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O43" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P43" s="5" t="inlineStr">
+        <is>
+          <t>An internally inconsistent specialist report (body citing one cause; associated quote describing a different remediation type) cannot establish EOW causation for damage beyond the confirmed area; salt contamination in walls is physical evidence of external water ingress inconsistent with internal EOW causation; policyholders must provide reliable, internally consistent expert evidence to extend an EOW claim beyond the confirmed damage area</t>
+        </is>
+      </c>
+      <c r="Q43" s="5" t="inlineStr">
+        <is>
+          <t>A follow-up expert report resolving the inconsistency between the damp specialist's attributed cause and the remediation description; independent assessment of whether the salt contamination pattern was consistent with EOW rather than external water ingress</t>
+        </is>
+      </c>
+      <c r="R43" s="5" t="inlineStr">
+        <is>
+          <t>The damp specialist report cited a persistent water leak in the body but described penetrating damp remediation in the quote — an internal inconsistency that undermined its reliability; salt contamination in the walls is physical evidence pointing to external water ingress rather than internal EOW; Aviva was entitled to limit coverage to the area where EOW causation was reliably established</t>
+        </is>
+      </c>
+      <c r="S43" s="5" t="inlineStr">
+        <is>
+          <t>When relying on a specialist report to extend an EOW claim, ensure the report is internally consistent between its attributed cause and its proposed remediation; salt contamination in walls is a key indicator of external water ingress that can defeat an EOW claim for that area; always obtain a follow-up report to resolve any inconsistency before submitting to FOS</t>
+        </is>
+      </c>
+      <c r="T43" s="5" t="inlineStr">
+        <is>
+          <t>IF specialist_report_body_cites_eow AND remediation_quote_describes_penetrating_damp THEN report = internally_inconsistent AND eow_causation_not_established; IF salt_contamination_in_walls THEN external_water_ingress_indicated AND eow_causation = weakened</t>
+        </is>
+      </c>
+      <c r="U43" s="4" t="inlineStr">
+        <is>
+          <t>DRN-5649220.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="120" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>EOW-043</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>DRN5670903</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Insurers at Lloyd's (Society of Lloyd's)</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>1 Mar 2020</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>Escape of water at an unfurnished residential property during a 5-day unfurnished period; insurer declined under a separate unfurnished property EOW exclusion distinct from the standard 30-day unoccupied exclusion</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>Escape of water during a period when the property was unfurnished (specific physical source not central to this decision)</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>Residential home (unfurnished at time of EOW — only 5 days)</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J44" s="3" t="inlineStr">
+        <is>
+          <t>Policy contained an endorsement excluding EOW cover where the property was unfurnished; property was unfurnished for 5 days at the time of the EOW; the unfurnished exclusion applied from day 1, before the 30-day unoccupied exclusion would have been triggered; insurer provided adequate justification for the higher risk</t>
+        </is>
+      </c>
+      <c r="K44" s="3" t="inlineStr">
+        <is>
+          <t>Policyholder argued 5 days unfurnished was unreasonably short to trigger the exclusion; insurer provided justification for the higher risk; FOS confirmed the unfurnished exclusion is distinct from and independent of the unoccupied exclusion</t>
+        </is>
+      </c>
+      <c r="L44" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M44" s="3" t="inlineStr">
+        <is>
+          <t>FOS did not uphold — the unfurnished endorsement applied from day 1; insurer provided adequate underwriting justification (higher risk when property is vacant and unfurnished, especially in winter); no award directed</t>
+        </is>
+      </c>
+      <c r="N44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O44" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P44" s="3" t="inlineStr">
+        <is>
+          <t>An unfurnished exclusion for EOW is legally distinct from an unoccupied exclusion; it applies from day 1 regardless of duration and before the 30-day unoccupied trigger; once an insurer provides adequate underwriting justification for the exclusion, FOS will not override it even if the period is very short; policyholders should note that unfurnished and unoccupied are separate policy conditions</t>
+        </is>
+      </c>
+      <c r="Q44" s="3" t="inlineStr">
+        <is>
+          <t>Specific policy wording of both the unfurnished endorsement and the 30-day unoccupied exclusion for comparison; evidence of whether the property had heating or other protective measures during the 5-day unfurnished period</t>
+        </is>
+      </c>
+      <c r="R44" s="3" t="inlineStr">
+        <is>
+          <t>The unfurnished endorsement is a separate and independent policy condition from the 30-day unoccupied exclusion; it applied from the moment the property became unfurnished, with no minimum period; the insurer provided adequate justification for the higher risk (vacant property in winter); FOS will not override a clearly worded and adequately justified underwriting decision</t>
+        </is>
+      </c>
+      <c r="S44" s="3" t="inlineStr">
+        <is>
+          <t>Always check for unfurnished endorsements specifically, as they operate independently of and are triggered earlier than standard unoccupied exclusions; where a property moves between furnished and unfurnished states, even briefly, the unfurnished endorsement may apply; document the property's furnishing status throughout the year if an unfurnished endorsement is in place</t>
+        </is>
+      </c>
+      <c r="T44" s="3" t="inlineStr">
+        <is>
+          <t>IF property_is_unfurnished AND policy_has_unfurnished_eow_exclusion THEN eow_exclusion = applies_from_day_1_regardless_of_duration; IF unfurnished_exclusion_present AND unoccupied_exclusion_present THEN they_are_independent_conditions</t>
+        </is>
+      </c>
+      <c r="U44" s="2" t="inlineStr">
+        <is>
+          <t>DRN5670903.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="120" customHeight="1">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>EOW-044</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>DRN-5805040</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>Saga Services Limited</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>8 Oct 2025</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>Escape of water at an estate property; Saga failed to disclose an endorsement change at renewal; insurer independently declined for breach of heating and drainage condition; counterfactual analysis showed alternative cover would also have excluded the loss</t>
+        </is>
+      </c>
+      <c r="F45" s="5" t="inlineStr">
+        <is>
+          <t>Escape of water during a period where heating and drainage condition was not met (specific physical source not the focus of this decision)</t>
+        </is>
+      </c>
+      <c r="G45" s="4" t="inlineStr">
+        <is>
+          <t>Residential home (property of deceased — executors)</t>
+        </is>
+      </c>
+      <c r="H45" s="4" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I45" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J45" s="5" t="inlineStr">
+        <is>
+          <t>Saga's primary defence was a heating and drainage endorsement that was not met at the time of the loss; independently, the endorsement had been changed at renewal without adequate disclosure; however, counterfactual analysis showed any alternative cover the policyholder would have purchased would also have contained equivalent heating and drainage requirements that were not met</t>
+        </is>
+      </c>
+      <c r="K45" s="5" t="inlineStr">
+        <is>
+          <t>Executors challenged the non-disclosure of the endorsement change at renewal; Saga relied on energy bill evidence to establish the heating condition was not met; executors argued smart meter data could challenge the energy bill evidence but did not obtain it; FOS found the counterfactual argument decisive</t>
+        </is>
+      </c>
+      <c r="L45" s="4" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M45" s="5" t="inlineStr">
+        <is>
+          <t>FOS did not uphold — even if the endorsement change should have been disclosed at renewal, alternative cover available to the policyholder would also have contained heating and drainage requirements that were not met; Saga's separate £1,250 goodwill offer was outside FOS jurisdiction; no FOS-directed award; FOS cannot award D&amp;I compensation to executors or estate representatives</t>
+        </is>
+      </c>
+      <c r="N45" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O45" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P45" s="5" t="inlineStr">
+        <is>
+          <t>Failure to disclose an endorsement change at renewal does not automatically result in coverage where counterfactual analysis shows the policyholder would not have obtained materially better cover elsewhere; FOS cannot award distress and inconvenience compensation to executors or estate representatives; a policyholder must produce positive evidence (e.g. smart meter data confirming billing errors) to challenge an insurer's documentary evidence of condition breach</t>
+        </is>
+      </c>
+      <c r="Q45" s="5" t="inlineStr">
+        <is>
+          <t>Smart meter data confirming an error in the energy bills used to establish the heating condition breach; evidence that alternative cover available at renewal would not have included an equivalent heating and drainage condition</t>
+        </is>
+      </c>
+      <c r="R45" s="5" t="inlineStr">
+        <is>
+          <t>The endorsement change non-disclosure was a valid complaint ground; however, even without the endorsement change, any equivalent cover the policyholder would have purchased would also have required compliance with heating and drainage conditions that were not met; the counterfactual analysis defeats the endorsement non-disclosure argument; energy bill evidence of condition breach was not successfully challenged; FOS cannot award D&amp;I compensation to estate representatives</t>
+        </is>
+      </c>
+      <c r="S45" s="5" t="inlineStr">
+        <is>
+          <t>Always conduct a counterfactual analysis when responding to non-disclosure of endorsement changes — if alternative cover would also have excluded the same loss, the non-disclosure argument fails; executors pursuing claims for deceased policyholders cannot receive D&amp;I compensation from FOS; challenge energy bill evidence of condition breaches with smart meter data at the earliest opportunity</t>
+        </is>
+      </c>
+      <c r="T45" s="5" t="inlineStr">
+        <is>
+          <t>IF insurer_failed_to_disclose_endorsement_change_at_renewal AND alternative_cover_would_also_exclude_same_loss THEN non_disclosure_argument = fails; IF complainant_is_executor_or_estate_representative THEN fos_di_compensation = NOT available</t>
+        </is>
+      </c>
+      <c r="U45" s="4" t="inlineStr">
+        <is>
+          <t>DRN-5805040.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="120" customHeight="1">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>EOW-045</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>DRN5927839</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Admiral Insurance (Gibraltar) Limited</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>18 May 2019</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>Escape of water in 2015 at a property already affected by dry rot; insurer declined citing gradual cause — dry rot requiring both wet timber and poor ventilation pre-existed the EOW; dominant cause (poor ventilation) not an insured peril</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>Escape of water (2015 event); ongoing damp; blocked air bricks; inadequate subfloor ventilation — multiple contributing factors</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J46" s="3" t="inlineStr">
+        <is>
+          <t>Dry rot requires both wet timber AND poor ventilation — both conditions pre-existed the claimed EOW; policyholders were notified of ongoing damp issues in 2015; the dominant cause of the dry rot outbreak was poor ventilation (blocked air bricks), not the EOW</t>
+        </is>
+      </c>
+      <c r="K46" s="3" t="inlineStr">
+        <is>
+          <t>Policyholders' expert argued a 2015 EOW caused the dry rot; Admiral's evidence showed both pre-conditions (wet timber and poor ventilation) pre-existed; expert who wrote the 2018 report gave contradictory views (written report vs subsequent email); FOS preferred the written report and found the gradual cause exclusion applied</t>
+        </is>
+      </c>
+      <c r="L46" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M46" s="3" t="inlineStr">
+        <is>
+          <t>FOS did not uphold — dry rot's dual preconditions (wet timber AND poor ventilation) both pre-existed; where the dominant cause (poor ventilation from blocked air bricks) is not an insured peril, Admiral's decline is sustainable; no award directed</t>
+        </is>
+      </c>
+      <c r="N46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O46" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P46" s="3" t="inlineStr">
+        <is>
+          <t>Dry rot requires both wet timber and poor ventilation; where both conditions pre-existed the claimed EOW event and the policyholder was notified of the conditions, the gradual cause exclusion applies even if the EOW contributed to one of those conditions; where the dominant cause of damage is not an insured peril (e.g. poor ventilation from blocked air bricks), the insurer's decline is sustainable; policyholders bear the burden of demonstrating the insured peril was the dominant cause</t>
+        </is>
+      </c>
+      <c r="Q46" s="3" t="inlineStr">
+        <is>
+          <t>Expert evidence establishing the precise chronology of when the dry rot developed relative to the EOW events; independent assessment definitively ruling out pre-existing dry rot before the 2015 EOW; consistent expert opinion</t>
+        </is>
+      </c>
+      <c r="R46" s="3" t="inlineStr">
+        <is>
+          <t>Both dry rot preconditions pre-existed the EOW; policyholders were notified of damp issues in 2015, establishing constructive knowledge; the expert's written report was preferred over the contradictory email; dominant cause analysis determined poor ventilation (blocked air bricks) was the primary cause — an uninsured peril; EOW's contribution to timber wetness does not make it the dominant cause</t>
+        </is>
+      </c>
+      <c r="S46" s="3" t="inlineStr">
+        <is>
+          <t>Dry rot claims involving EOW require analysis of all preconditions for dry rot (wet timber AND poor ventilation); where both pre-existed and the policyholder had notice of damp, the gradual cause exclusion is strong; dominant cause analysis is key — establish which condition was the primary driver of the rot; written expert reports are given more weight than subsequent conflicting oral or email communications</t>
+        </is>
+      </c>
+      <c r="T46" s="3" t="inlineStr">
+        <is>
+          <t>IF dry_rot_claimed AND both_preconditions_preexisted AND policyholder_notified_of_damp THEN gradual_cause_exclusion = applicable; IF dominant_cause_is_uninsured_peril THEN eow_contribution = insufficient_for_coverage</t>
+        </is>
+      </c>
+      <c r="U46" s="2" t="inlineStr">
+        <is>
+          <t>DRN5927839.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="120" customHeight="1">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>EOW-046</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>DRN-5979060</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>Ecclesiastical Insurance Office Plc</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>19 Jan 2026</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>Second FOS complaint about reinstatement scope following a March 2024 FOS direction; dispute about whether undersized joists causing floor deflection were damaged by EOW or were a pre-existing structural issue</t>
+        </is>
+      </c>
+      <c r="F47" s="5" t="inlineStr">
+        <is>
+          <t>Escape of water (specific source addressed in prior FOS decision — this decision concerns follow-on expert assessment of specific structural components)</t>
+        </is>
+      </c>
+      <c r="G47" s="4" t="inlineStr">
+        <is>
+          <t>Residential home (holiday home)</t>
+        </is>
+      </c>
+      <c r="H47" s="4" t="inlineStr">
+        <is>
+          <t>Handling / Reinstatement Dispute</t>
+        </is>
+      </c>
+      <c r="I47" s="4" t="inlineStr">
+        <is>
+          <t>Accepted — Disputed Settlement</t>
+        </is>
+      </c>
+      <c r="J47" s="5" t="inlineStr">
+        <is>
+          <t>Following the March 2024 FOS direction to reconsider, Ecclesiastical appointed a suitably qualified expert who found the floor deflection (undersized joists) was a structural issue independent of the EOW; insurer declined to include joist replacement in the scope</t>
+        </is>
+      </c>
+      <c r="K47" s="5" t="inlineStr">
+        <is>
+          <t>Policyholder relied on photographs to argue the joists were damaged by EOW; Ecclesiastical's qualified expert (appointed pursuant to the prior FOS direction) found undersized joists causing floor deflection is a pre-existing structural issue independent of the EOW event; FOS preferred the expert's structured physical assessment over the policyholder's photographs</t>
+        </is>
+      </c>
+      <c r="L47" s="4" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M47" s="5" t="inlineStr">
+        <is>
+          <t>FOS did not uphold — Ecclesiastical had complied with the prior FOS direction by appointing a suitably qualified expert; that expert's findings that the joist issue was structural and pre-existing were reliable and reasonable; policyholder photographs alone were insufficient to override a structured expert report; no further award directed</t>
+        </is>
+      </c>
+      <c r="N47" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O47" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P47" s="5" t="inlineStr">
+        <is>
+          <t>Where an insurer appoints a suitably qualified expert pursuant to a prior FOS direction and that expert finds a specific component's problem is structural and pre-existing and independent of the EOW, the insurer has discharged its obligation under the FOS direction; policyholder photographs alone are insufficient to override the findings of a structured expert physical assessment; compliance with a prior FOS direction is assessed by reference to the quality of the process, not whether the outcome favours the policyholder</t>
+        </is>
+      </c>
+      <c r="Q47" s="5" t="inlineStr">
+        <is>
+          <t>Independent structural engineer assessment of the joist condition both before and after the EOW event; photographic evidence taken closer to the time of the EOW showing the joist condition at that point</t>
+        </is>
+      </c>
+      <c r="R47" s="5" t="inlineStr">
+        <is>
+          <t>Ecclesiastical complied with the prior FOS direction by appointing a qualified expert; that expert conducted a physical assessment and found the joist deflection was caused by undersized joists — a structural issue pre-existing the EOW; the policyholder's photographs did not constitute expert evidence capable of overriding a structured assessment; FOS would not require Ecclesiastical to take further action on a properly investigated structural finding</t>
+        </is>
+      </c>
+      <c r="S47" s="5" t="inlineStr">
+        <is>
+          <t>Compliance with a FOS direction to reconsider requires appointing a suitably qualified expert and properly documenting their findings; a structured expert physical assessment will take precedence over policyholder photographs; where a prior FOS complaint resulted in a direction, document the expert appointment and methodology carefully to demonstrate compliance</t>
+        </is>
+      </c>
+      <c r="T47" s="5" t="inlineStr">
+        <is>
+          <t>IF fos_direction_issued_to_reconsider AND insurer_appoints_qualified_expert AND expert_finds_no_eow_damage THEN insurer_complied_with_direction; IF policyholder_relies_only_on_photographs AND insurer_has_structured_expert_report THEN expert_report = more_persuasive</t>
+        </is>
+      </c>
+      <c r="U47" s="4" t="inlineStr">
+        <is>
+          <t>DRN-5979060.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="120" customHeight="1">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>EOW-047</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>DRN-5982848</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Protector Insurance UK</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>24 Mar 2026</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>Escape of water at a leasehold flat in a council-managed block; kitchen EOW damage accepted but bathroom and hallway damage and pre-EOW electrical works declined; dispute about causation of bathroom and hallway damage</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>Escape of water causing kitchen damage; bathroom damage attributed to steam and insufficient ventilation; hallway mould attributed to condensation; pre-EOW electrical works confirmed by rewiring quotation obtained before the EOW</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>Leasehold flat (block policy with council as freeholder)</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>Accepted — Disputed Settlement</t>
+        </is>
+      </c>
+      <c r="J48" s="3" t="inlineStr">
+        <is>
+          <t>Inspection report identified bathroom ceiling paint peeling consistent with steam and insufficient ventilation (not EOW); hallway mould consistent with condensation; pre-EOW rewiring quotation confirmed electrical works were pre-existing; loss adjuster's report considered valid basis for partial decline</t>
+        </is>
+      </c>
+      <c r="K48" s="3" t="inlineStr">
+        <is>
+          <t>Policyholder argued bathroom and hallway damage was caused by the EOW; inspection report showed evidence of steam damage and condensation rather than water ingress from EOW; pre-EOW rewiring quotation was contemporaneous evidence of pre-existing electrical issue; loss adjuster conducted a physical site inspection — considered as valid as a surveyor's report</t>
+        </is>
+      </c>
+      <c r="L48" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M48" s="3" t="inlineStr">
+        <is>
+          <t>FOS did not uphold the disputed elements — bathroom damage consistent with steam and insufficient ventilation, not EOW; hallway mould consistent with condensation, not EOW; pre-EOW rewiring quotation established electrical works were pre-existing; kitchen EOW damage accepted as confirmed</t>
+        </is>
+      </c>
+      <c r="N48" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O48" s="2" t="inlineStr">
+        <is>
+          <t>No — Commercial</t>
+        </is>
+      </c>
+      <c r="P48" s="3" t="inlineStr">
+        <is>
+          <t>Where an inspection report identifies damage patterns consistent with steam or condensation rather than EOW, insurer may decline those specific areas while accepting confirmed EOW damage elsewhere; a pre-EOW rewiring quotation is strong contemporaneous evidence that electrical works were pre-existing; a loss adjuster's physical site inspection report carries equal evidential weight to a surveyor's report</t>
+        </is>
+      </c>
+      <c r="Q48" s="3" t="inlineStr">
+        <is>
+          <t>Independent assessment distinguishing between EOW-caused moisture and steam and condensation damage in the bathroom; evidence of the ventilation conditions in the bathroom and hallway at the time of the EOW</t>
+        </is>
+      </c>
+      <c r="R48" s="3" t="inlineStr">
+        <is>
+          <t>The inspection report's observations (peeling paint consistent with steam; mould consistent with condensation) supported the partial decline; the pre-EOW rewiring quotation was contemporaneous and compelling evidence that the electrical damage preceded the EOW; a loss adjuster with physical site access is qualified to make causation assessments; kitchen EOW damage was separately confirmed and accepted</t>
+        </is>
+      </c>
+      <c r="S48" s="3" t="inlineStr">
+        <is>
+          <t>Always check whether bathroom damage patterns (peeling ceiling paint, mould) are more consistent with steam or condensation than EOW — these require different causation evidence; a pre-EOW contractor quotation is strong evidence of pre-existing works; loss adjuster reports carry equal weight to surveyor reports where a physical inspection was performed</t>
+        </is>
+      </c>
+      <c r="T48" s="3" t="inlineStr">
+        <is>
+          <t>IF bathroom_ceiling_paint_peeling AND consistent_with_steam_not_eow THEN bathroom_damage = NOT eow_caused; IF pre_eow_contractor_quotation_obtained THEN works_described = pre_existing; IF loss_adjuster_conducted_physical_inspection THEN report = as_valid_as_surveyor_report</t>
+        </is>
+      </c>
+      <c r="U48" s="2" t="inlineStr">
+        <is>
+          <t>DRN-5982848.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="120" customHeight="1">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>EOW-048</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>DRN-6004362</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>Aviva Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>14 Jan 2026</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>Escape of water from a burst water pipe; claim accepted December 2022 but not progressed for over 2 years; dispute about handling delays, settlement quantum, and contractor options</t>
+        </is>
+      </c>
+      <c r="F49" s="5" t="inlineStr">
+        <is>
+          <t>Burst water pipe (December 2022)</t>
+        </is>
+      </c>
+      <c r="G49" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H49" s="4" t="inlineStr">
+        <is>
+          <t>Handling / Reinstatement Dispute</t>
+        </is>
+      </c>
+      <c r="I49" s="4" t="inlineStr">
+        <is>
+          <t>Accepted — Disputed Settlement</t>
+        </is>
+      </c>
+      <c r="J49" s="5" t="inlineStr">
+        <is>
+          <t>N/A — claim accepted; Aviva failed to arrange an inspection for over 2 years; the eventual cash settlement (~£5,000 based on expert scope) was significantly lower than Mr R's own estimate; Mr R also disputed whether Aviva had offered contractor repairs</t>
+        </is>
+      </c>
+      <c r="K49" s="5" t="inlineStr">
+        <is>
+          <t>Aviva relied on independent engineer's inspection report and costed scope of works for the cash settlement; Mr R had no independent expert report contradicting those findings; additional correspondence produced by Aviva demonstrated the contractor option was offered on multiple occasions (January 2024, February 2025, June 2025, December 2025); Mr R's assertion of no contractor offer was not supported by the evidence</t>
+        </is>
+      </c>
+      <c r="L49" s="4" t="inlineStr">
+        <is>
+          <t>Upheld in Part</t>
+        </is>
+      </c>
+      <c r="M49" s="5" t="inlineStr">
+        <is>
+          <t>FOS upheld in part — Aviva directed to pay £750 total compensation (£300 already offered plus £450 additional) for failure to progress the claim proactively; Aviva to offer Mr R the option of their own contractors completing repairs; if Mr R declines contractor option, cash settlement per the expert scope to be paid; if additional EOW-related damage found during repairs, Aviva to consider it under the policy</t>
+        </is>
+      </c>
+      <c r="N49" s="4" t="n">
+        <v>750</v>
+      </c>
+      <c r="O49" s="4" t="inlineStr">
+        <is>
+          <t>No — Handling Dispute</t>
+        </is>
+      </c>
+      <c r="P49" s="5" t="inlineStr">
+        <is>
+          <t>The onus is on the insurer to progress an accepted claim proactively even where the policyholder prefers to self-source contractors; an insurer is entitled to rely on an independent expert's scope and costing as the basis for settlement where no contradictory expert opinion is produced; where a policyholder declined a contractor option and chose self-sourcing, the insurer's responsibility for resulting delays is reduced; FOS will not re-underwrite the quantum of a settlement based on an unchallenged expert report</t>
+        </is>
+      </c>
+      <c r="Q49" s="5" t="inlineStr">
+        <is>
+          <t>No independent expert report from Mr R contradicting the scope and costings; clear documented evidence of when the contractor option was offered (eventually produced and accepted as evidence of three separate offers)</t>
+        </is>
+      </c>
+      <c r="R49" s="5" t="inlineStr">
+        <is>
+          <t>Aviva accepted the claim in December 2022 but did not arrange inspection until April 2025 — over 2 years; despite this, Mr R was offered the contractor option multiple times and chose to self-source; shared responsibility for delays reduced the compensation from an initial £1,300 to £750; settlement based on the unchallenged expert report was fair; contractor option must be formally re-offered</t>
+        </is>
+      </c>
+      <c r="S49" s="5" t="inlineStr">
+        <is>
+          <t>Accepted EOW claims must be progressed proactively by the insurer even where a policyholder is self-sourcing contractors; offer the contractor repair option in writing and retain documentary evidence of each offer; where no contradictory expert report is produced, FOS will uphold a settlement based on the insurer's own expert scope; shared responsibility for delays significantly reduces compensation</t>
+        </is>
+      </c>
+      <c r="T49" s="5" t="inlineStr">
+        <is>
+          <t>IF accepted_claim_not_progressed_2_years AND insurer_did_offer_contractors AND policyholder_chose_self_sourcing THEN shared_responsibility = true AND compensation = reduced; IF no_contradictory_expert_report THEN insurer_settlement_based_on_own_expert = upheld</t>
+        </is>
+      </c>
+      <c r="U49" s="4" t="inlineStr">
+        <is>
+          <t>DRN-6004362.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="120" customHeight="1">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>EOW-049</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>DRN-6046762</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>INTACT INSURANCE UK LIMITED</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>27 Jan 2026</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>Escape of water at a residential property; claim accepted subject to average (underinsurance); dispute about five specific settlement points — drying costs subject to average, survey reimbursement, quote inflation, chimney inspection, Christmas food spoilage</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>Escape of water (specific source not central to this decision — dispute concerns settlement terms on an accepted claim)</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>Handling / Reinstatement Dispute</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>Accepted — Disputed Settlement</t>
+        </is>
+      </c>
+      <c r="J50" s="3" t="inlineStr">
+        <is>
+          <t>Claim settled subject to average (underinsurance); RSA applied average to all claim-related costs including drying invoice; declined full survey reimbursement; attributed quote inflation to policyholder's delay; declined chimney specialist inspection as no evidence of EOW damage; declined food spoilage as kitchen undamaged and property not evacuated</t>
+        </is>
+      </c>
+      <c r="K50" s="3" t="inlineStr">
+        <is>
+          <t>(1) Drying invoice — RSA applied average to all costs including monitoring and certificates; FOS confirmed these are claim-related and correctly subject to average; (2) Survey costs — RSA offered £90 of £360; FOS could not find on this as underinsurance position excluded from scope; (3) Quote inflation — 1.76% attributed to Miss J's delay in providing own survey; FOS found RSA's approach fair; (4) Chimney — loss adjuster found no evidence of EOW damage; (5) Christmas food £50 — kitchen undamaged and no evacuation needed</t>
+        </is>
+      </c>
+      <c r="L50" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M50" s="3" t="inlineStr">
+        <is>
+          <t>FOS did not uphold any of the five disputed points — all aspects of RSA's settlement approach were reasonable and fair; no further payment directed</t>
+        </is>
+      </c>
+      <c r="N50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O50" s="2" t="inlineStr">
+        <is>
+          <t>No — Handling Dispute</t>
+        </is>
+      </c>
+      <c r="P50" s="3" t="inlineStr">
+        <is>
+          <t>All claim-related costs on an underinsured claim (including drying survey fees, certificates and monitoring) are properly subject to average; a policyholder who delays providing their own survey bears responsibility for resulting quote inflation; a loss adjuster conducting a physical inspection is qualified to assess whether a specific component was damaged by EOW; food spoilage is not covered where the kitchen is undamaged and no evacuation was required</t>
+        </is>
+      </c>
+      <c r="Q50" s="3" t="inlineStr">
+        <is>
+          <t>Evidence of whether the survey delay was attributable to RSA or the policyholder; independent chimney specialist report linking chimney damage to EOW; compelling evidence linking food disposal directly to the EOW rather than the claimant's own decision</t>
+        </is>
+      </c>
+      <c r="R50" s="3" t="inlineStr">
+        <is>
+          <t>Drying costs are claim costs subject to average regardless of their specific nature; survey cost finding was precluded as the underinsurance position was outside scope; quote inflation arose from Miss J's own delay in commissioning and providing the survey; loss adjuster found no EOW chimney damage and is qualified to make that assessment; no compelling reason why the EOW caused food to be thrown away where the kitchen was undamaged and the property was not evacuated</t>
+        </is>
+      </c>
+      <c r="S50" s="3" t="inlineStr">
+        <is>
+          <t>On underinsured claims, all claim-related costs — including specialist monitoring and certification fees — are subject to average; policyholders must be clearly advised at the outset to provide required documentation promptly to avoid bearing quote inflation risk; where a loss adjuster conducts a physical inspection and finds no EOW damage, no specialist inspection obligation arises; ancillary loss claims (food, minor spoilage) require a clear causal link to the EOW</t>
+        </is>
+      </c>
+      <c r="T50" s="3" t="inlineStr">
+        <is>
+          <t>IF claim_subject_to_average AND drying_invoice_includes_monitoring_fees THEN monitoring_fees = subject_to_average; IF policyholder_delays_own_survey AND quote_inflation_results THEN policyholder_bears_inflation_cost; IF loss_adjuster_physical_inspection_finds_no_eow_damage THEN no_specialist_inspection_required</t>
+        </is>
+      </c>
+      <c r="U50" s="2" t="inlineStr">
+        <is>
+          <t>DRN-6046762.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="120" customHeight="1">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>EOW-050</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>DRN6187392</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>St Andrew's Insurance Plc</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="inlineStr"/>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>Floor cracking attributed by insurer to sulphate attack from water exposure; initially presented as heave and subsidence claim; FOS directed insurer to investigate under EOW cover based on its own causation explanation</t>
+        </is>
+      </c>
+      <c r="F51" s="5" t="inlineStr">
+        <is>
+          <t>Disputed — St Andrew's attributed floor cracking to sulphate attack caused by water exposure (potentially from damp ground, fill material, or EOW); origin of the water not determined</t>
+        </is>
+      </c>
+      <c r="G51" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H51" s="4" t="inlineStr">
+        <is>
+          <t>Peril Classification Dispute</t>
+        </is>
+      </c>
+      <c r="I51" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J51" s="5" t="inlineStr">
+        <is>
+          <t>St Andrew's declined under heave and subsidence — no heave of the site (only floor movement); also argued exclusion for solid floor movement without concurrent foundation damage; both grounds found partially deficient by FOS</t>
+        </is>
+      </c>
+      <c r="K51" s="5" t="inlineStr">
+        <is>
+          <t>St Andrew's relied on its expert's opinion that no site heave occurred and the floor movement exclusion applied; Miss F's representative (retired engineer) argued site investigations were needed; FOS found the sulphate attack explanation itself created a sufficient factual basis for an EOW investigation; FOS also found St Andrew's had not adequately justified the foundations exclusion</t>
+        </is>
+      </c>
+      <c r="L51" s="4" t="inlineStr">
+        <is>
+          <t>Upheld in Part</t>
+        </is>
+      </c>
+      <c r="M51" s="5" t="inlineStr">
+        <is>
+          <t>FOS upheld in part — St Andrew's Insurance Plc directed to consider the damage under EOW cover in accordance with policy terms and FOS guidance; if heave of the site is later established, St Andrew's to consider under that cover without reference to the foundations exclusion; no monetary award</t>
+        </is>
+      </c>
+      <c r="N51" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O51" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P51" s="5" t="inlineStr">
+        <is>
+          <t>Where an insurer's own explanation for floor damage (sulphate attack caused by water exposure) is consistent with an EOW cause, that explanation creates sufficient grounds for an EOW investigation; but-for causation — if EOW caused the sulphate attack, the insurer cannot dismiss liability by pointing to the sulphate attack as the proximate cause; an insurer seeking to rely on a foundations exclusion must provide specific reasoning for why foundations are unaffected, not merely assert it</t>
+        </is>
+      </c>
+      <c r="Q51" s="5" t="inlineStr">
+        <is>
+          <t>Investigation results confirming or ruling out an EOW below the floor; evidence that the foundation external walls were or were not also affected by the same process; clear photographic record of the crack to external render cited by Mr J</t>
+        </is>
+      </c>
+      <c r="R51" s="5" t="inlineStr">
+        <is>
+          <t>St Andrew's own explanation (sulphate attack from water) is consistent with an EOW origin — this shifts the burden to St Andrew's to demonstrate no EOW occurred or a valid exclusion applies; St Andrew's did not acknowledge the crack in external render cited by Mr J, let alone explain why it was irrelevant to the foundations exclusion; FOS directed EOW investigation as the appropriate next step</t>
+        </is>
+      </c>
+      <c r="S51" s="5" t="inlineStr">
+        <is>
+          <t>When an insurer's own damage explanation involves water exposure that is consistent with an EOW cause, the insurer must investigate under EOW cover; but-for causation applies to the EOW pathway — do not simply pass liability to the secondary mechanism (sulphate attack); when invoking a foundations exclusion, provide specific reasons why foundations are unaffected with reference to all physical evidence including any cracks noted by the policyholder</t>
+        </is>
+      </c>
+      <c r="T51" s="5" t="inlineStr">
+        <is>
+          <t>IF insurer_attributes_damage_to_sulphate_attack_from_water AND eow_is_plausible_water_source THEN insurer_must_investigate_under_eow_cover; IF insurer_relies_on_foundations_exclusion AND has_not_addressed_visible_cracks_near_foundations THEN exclusion_justification = insufficient</t>
+        </is>
+      </c>
+      <c r="U51" s="4" t="inlineStr">
+        <is>
+          <t>DRN6187392.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="120" customHeight="1">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>EOW-051</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>DRN-6263959</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Tesco Underwriting Limited</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>28 Apr 2026</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>Kitchen ceiling leak identified by home emergency provider; ceiling damage claimed under home insurance trace and access section; insurer applied the higher EOW section excess rather than the lower trace and access excess</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>Leak in ceiling above kitchen; identified and fixed by home emergency contractor under separate home emergency policy</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>Handling / Reinstatement Dispute</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>Accepted — Disputed Settlement</t>
+        </is>
+      </c>
+      <c r="J52" s="3" t="inlineStr">
+        <is>
+          <t>Tesco applied the EOW section excess (£350 compulsory plus £200 voluntary = £550) rather than the trace and access section excess, on the basis that some water damage existed before the trace and access work; FOS found the damage was confined to the trace and access area and T&amp;A classification was fairer</t>
+        </is>
+      </c>
+      <c r="K52" s="3" t="inlineStr">
+        <is>
+          <t>Tesco relied on pre-existing staining and cracking in photographs to support an EOW classification; FOS examined photographs taken after the ceiling was cut for trace and access work and found damage was confined to the same small area; ceiling was in good condition with no widespread water damage consistent with EOW; repair work would be identical regardless of which section applied</t>
+        </is>
+      </c>
+      <c r="L52" s="2" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M52" s="3" t="inlineStr">
+        <is>
+          <t>Tesco Underwriting Limited directed to pay Mr H £250 to refund the excess differential (or pay a net settlement of £530 if no settlement yet made); claim to be processed under trace and access section at the lower excess</t>
+        </is>
+      </c>
+      <c r="N52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O52" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P52" s="3" t="inlineStr">
+        <is>
+          <t>Where damage is confined to the trace and access work area and photographs show no widespread water damage, it is fairer and more pragmatic to settle under the trace and access section even if an EOW event technically occurred; an insurer cannot use EOW peril classification to impose a materially higher excess where both sections would produce identical repair costs; policyholders are entitled to claim under the policy section most beneficial to them where multiple sections could apply to the same facts</t>
+        </is>
+      </c>
+      <c r="Q52" s="3" t="inlineStr">
+        <is>
+          <t>Evidence of widespread pre-existing water damage (tidemarks, widespread staining) beyond the trace and access work area; photographs taken before the trace and access work showing the ceiling condition</t>
+        </is>
+      </c>
+      <c r="R52" s="3" t="inlineStr">
+        <is>
+          <t>Photographs taken after the T&amp;A access cut showed damage confined to a small area consistent with T&amp;A work — no frayed edges, no widespread water damage patterns; applying the T&amp;A section would produce identical repair work and costs; Tesco should not use EOW classification to impose a higher excess where damage was localised; £250 excess differential to be refunded or credited</t>
+        </is>
+      </c>
+      <c r="S52" s="3" t="inlineStr">
+        <is>
+          <t>When settling a claim involving both T&amp;A and potential EOW elements, check photographs for evidence of widespread water damage beyond the T&amp;A area; if damage is confined to the T&amp;A area, the T&amp;A section should be used; always apply the policy section most beneficial to the policyholder where both apply to the same facts</t>
+        </is>
+      </c>
+      <c r="T52" s="3" t="inlineStr">
+        <is>
+          <t>IF damage_confined_to_ta_access_area AND no_widespread_water_damage_in_photographs THEN ta_section_classification = appropriate AND lower_excess_applies; IF two_policy_sections_applicable AND repair_costs_identical THEN use_section_most_beneficial_to_policyholder</t>
+        </is>
+      </c>
+      <c r="U52" s="2" t="inlineStr">
+        <is>
+          <t>DRN-6263959.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="120" customHeight="1">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>EOW-052</t>
+        </is>
+      </c>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>DRN6739737</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>Royal &amp; Sun Alliance Insurance Plc</t>
+        </is>
+      </c>
+      <c r="D53" s="4" t="inlineStr">
+        <is>
+          <t>6 Jan 2020</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>Cracking floor tiles at residential property; policyholder suspected EOW; RSA's surveyor found no evidence of EOW and attributed cracking to poorly fitted subfloor boards; RSA declined to carry out trace and access investigation</t>
+        </is>
+      </c>
+      <c r="F53" s="5" t="inlineStr">
+        <is>
+          <t>Disputed — no EOW confirmed; RSA's surveyor attributed cracking to chipboard and plywood subfloor boards not securely fixed, expanding when the house heats up</t>
+        </is>
+      </c>
+      <c r="G53" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H53" s="4" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I53" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J53" s="5" t="inlineStr">
+        <is>
+          <t>No evidence of an escape of water or any other insurable event; RSA's surveyor attributed floor tile cracking to poor workmanship (inadequately fixed subfloor boards); without an established insured event, trace and access cover was not triggered under the policy wording</t>
+        </is>
+      </c>
+      <c r="K53" s="5" t="inlineStr">
+        <is>
+          <t>Miss M relied on a civil engineer's recommendation for further intrusive investigations and claimed the RSA inspector told her trace and access should apply; RSA relied on its surveyor's report finding no EOW and an alternative workmanship explanation; policy wording required evidence of an EOW before T&amp;A cover applied; FOS read the surveyor's own notes as directing Miss M to carry out T&amp;A if she chose, not as an insurer obligation</t>
+        </is>
+      </c>
+      <c r="L53" s="4" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M53" s="5" t="inlineStr">
+        <is>
+          <t>FOS did not uphold — trace and access cover was not triggered without confirmed evidence of an EOW insured event; RSA's surveyor's alternative explanation was reasonable; if Miss M later funds exploratory works and an EOW is confirmed, RSA stated it would consider a claim in line with policy terms; no further action required</t>
+        </is>
+      </c>
+      <c r="N53" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O53" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P53" s="5" t="inlineStr">
+        <is>
+          <t>Trace and access cover is triggered by confirmed evidence of an escape of water, not by a suspected or possible EOW; where an insurer's surveyor provides an alternative non-EOW explanation for damage with expert support, the insurer is not required to fund intrusive investigations; the policyholder may self-fund exploratory works and submit a claim if an EOW is subsequently confirmed; surveyor's notes recommending T&amp;A as an option for the policyholder are not the same as an insurer commitment to fund T&amp;A</t>
+        </is>
+      </c>
+      <c r="Q53" s="5" t="inlineStr">
+        <is>
+          <t>Intrusive investigation results confirming whether an EOW had occurred beneath the floor tiles; independent expert refuting RSA's surveyor's alternative workmanship explanation</t>
+        </is>
+      </c>
+      <c r="R53" s="5" t="inlineStr">
+        <is>
+          <t>Policy wording required evidence of an EOW for T&amp;A cover to apply; RSA's surveyor provided a credible non-EOW explanation; civil engineer's recommendation for further investigation did not establish that an EOW had occurred; surveyor's paper note directing Miss M to carry out T&amp;A was addressed to Miss M as an option, not as an insurer commitment; T&amp;A is available once an EOW is confirmed</t>
+        </is>
+      </c>
+      <c r="S53" s="5" t="inlineStr">
+        <is>
+          <t>Trace and access cover requires established evidence of an EOW — suspected or possible EOW is not sufficient to trigger T&amp;A; where an insurer's surveyor identifies a plausible non-EOW cause for floor damage, the insurer may decline without further investigation; advise policyholders clearly that they may self-fund exploratory works and claim if an EOW is found</t>
+        </is>
+      </c>
+      <c r="T53" s="5" t="inlineStr">
+        <is>
+          <t>IF no_evidence_of_eow AND alternative_non_eow_explanation_established THEN ta_cover = NOT triggered; IF policyholder_suspects_eow AND insurer_surveyor_finds_no_eow THEN insurer_not_required_to_fund_ta_investigations</t>
+        </is>
+      </c>
+      <c r="U53" s="4" t="inlineStr">
+        <is>
+          <t>DRN6739737.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="120" customHeight="1">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>EOW-053</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>DRN7090448</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>UK Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>19 Jan 2015</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>Escape of water from neighbour's bath overflow entering a rental property between tenancies; insurer declined under vacancy exclusion (30+ days unoccupied); ceiling collapsed on day 34 suggesting progressive ingress began before the 30-day period expired</t>
+        </is>
+      </c>
+      <c r="F54" s="3" t="inlineStr">
+        <is>
+          <t>Neighbour's bath overflow (overflow fault requiring a plumber to fix — not a tap left running); water entered through ceiling from above property</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>Residential home (rental property, tenants vacated 33 days before discovery)</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J54" s="3" t="inlineStr">
+        <is>
+          <t>UKI invoked the vacancy exclusion — property unoccupied, untenanted or not actively used for more than 30 consecutive days; tenants had vacated 33 days before the water was noticed; UKI concluded the escape of water occurred after the 30-day period expired</t>
+        </is>
+      </c>
+      <c r="K54" s="3" t="inlineStr">
+        <is>
+          <t>UKI relied on the 33-day vacancy period and stated the escape of water was due to a bath overflow discovered on the date of occurrence; Mr K argued the ceiling collapse on day 34 was evidence that water ingress had been occurring over several days — inconsistent with a single-day event; the neighbour called a plumber to fix the overflow, suggesting a pipe or overflow fault rather than a tap left running</t>
+        </is>
+      </c>
+      <c r="L54" s="2" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M54" s="3" t="inlineStr">
+        <is>
+          <t>UK Insurance Limited directed to reconsider Mr K's claim in line with the remaining policy terms and conditions; pay £200 compensation for inconvenience caused by the handling of the claim; reissue expired £24 cheque previously paid for initial customer service failure</t>
+        </is>
+      </c>
+      <c r="N54" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="O54" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P54" s="3" t="inlineStr">
+        <is>
+          <t>An insurer invoking a vacancy exclusion must demonstrate on the balance of probabilities that the escape of water actually occurred after the vacancy trigger period expired — the date damage was noticed is not determinative; ceiling collapse on the day after discovery suggests progressive water ingress over multiple days starting before the 30-day mark; where a neighbour calls a plumber to fix an overflow, this is consistent with a pipe fault that may have been leaking for days rather than a single tap-on event</t>
+        </is>
+      </c>
+      <c r="Q54" s="3" t="inlineStr">
+        <is>
+          <t>Plumber's report confirming when the overflow fault began and how long it may have been present; inspection of the neighbour's bathroom at the time to establish the nature of the overflow fault</t>
+        </is>
+      </c>
+      <c r="R54" s="3" t="inlineStr">
+        <is>
+          <t>If the escape of water was simply a tap left running, no plumber would be needed to fix it — the fact a plumber was called suggests an overflow fault that had been developing; ceiling collapse on day 34 is inconsistent with a single-day water ingress event and more consistent with progressive ingress over days; UKI did not demonstrate that the escape of water started after the 30-day vacancy period expired; EOW more likely began before the 30-day period ended</t>
+        </is>
+      </c>
+      <c r="S54" s="3" t="inlineStr">
+        <is>
+          <t>When invoking a vacancy exclusion for EOW, analyse the physical evidence of water ingress duration (e.g. degree of ceiling collapse, saturation levels) to determine whether the EOW more likely started before or after the vacancy trigger; a neighbour requiring a plumber to fix an overflow suggests a pipe fault rather than a single negligent act, increasing the likelihood of progressive ingress starting earlier</t>
+        </is>
+      </c>
+      <c r="T54" s="3" t="inlineStr">
+        <is>
+          <t>IF vacancy_exclusion_invoked AND ceiling_collapsed_day_after_discovery THEN progressive_ingress_likely_started_before_vacancy_period AND exclusion = NOT established; IF neighbour_called_plumber_to_fix_overflow THEN overflow_fault_not_single_event AND earlier_start_date = more_probable</t>
+        </is>
+      </c>
+      <c r="U54" s="2" t="inlineStr">
+        <is>
+          <t>DRN7090448.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="120" customHeight="1">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>EOW-054</t>
+        </is>
+      </c>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>DRN7112734</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t>Hiscox Insurance Company Limited</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr"/>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>EOW from drains caused sub-soil washout and building subsidence; claim settled and paid by Hiscox; dispute about whether the claim should be recorded as EOW or subsidence for future renewal and premium purposes</t>
+        </is>
+      </c>
+      <c r="F55" s="5" t="inlineStr">
+        <is>
+          <t>Escape of water from drains — caused sub-soil to be washed away, leading to downward movement of the site and cracking of building walls</t>
+        </is>
+      </c>
+      <c r="G55" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H55" s="4" t="inlineStr">
+        <is>
+          <t>Claim Recording / Administrative Dispute</t>
+        </is>
+      </c>
+      <c r="I55" s="4" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="J55" s="5" t="inlineStr">
+        <is>
+          <t>N/A — claim was settled and paid by Hiscox under the EOW excess; post-settlement, Hiscox recorded the claim as subsidence for renewal and database purposes; Miss A disputed this recording</t>
+        </is>
+      </c>
+      <c r="K55" s="5" t="inlineStr">
+        <is>
+          <t>Miss A relied on the settlement form headed Escape of Water and the use of an EOW excess to argue the claim was recorded as EOW; Hiscox argued escape of water on the settlement form referred to the applicable excess rate, not the claim category; engineer's own report stated damage consistent with a recent episode of subsidence and recommended applying the EOW excess; FOS agreed with Hiscox's characterisation of the settlement form</t>
+        </is>
+      </c>
+      <c r="L55" s="4" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M55" s="5" t="inlineStr">
+        <is>
+          <t>FOS did not uphold — the physical damage (downward movement of site and cracking) was correctly characterised as subsidence regardless of the water trigger mechanism; Hiscox's use of escape of water on the settlement form related only to the applicable excess rate; no award directed; Miss A not entitled to have the record changed or to premium refund</t>
+        </is>
+      </c>
+      <c r="N55" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O55" s="4" t="inlineStr">
+        <is>
+          <t>No — Administrative</t>
+        </is>
+      </c>
+      <c r="P55" s="5" t="inlineStr">
+        <is>
+          <t>The category of a claim is determined by the nature of the physical damage to the insured property, not by the mechanism that triggered that damage; where EOW from drains caused sub-soil washout leading to site movement and building cracking, the physical damage is subsidence in nature; where a settlement form uses escape of water in the context of applying a lower policy excess, this refers to the excess applicable — not to the claim category for recording purposes</t>
+        </is>
+      </c>
+      <c r="Q55" s="5" t="inlineStr">
+        <is>
+          <t>Evidence from the loss adjuster or engineer establishing exactly how the settlement form's use of escape of water was intended; premium comparison data showing whether Miss A paid higher premiums due to the subsidence record</t>
+        </is>
+      </c>
+      <c r="R55" s="5" t="inlineStr">
+        <is>
+          <t>Engineer stated damage was consistent with a recent episode of subsidence — the EOW from drains was the mechanism but subsidence was the resulting physical damage type; escape of water on the settlement form referred to applying the lower EOW excess rather than categorising the claim as EOW; throughout correspondence, subsidence was the consistent terminology used; the neighbour's insurer categorising the same event as EOW does not compel Hiscox to do the same</t>
+        </is>
+      </c>
+      <c r="S55" s="5" t="inlineStr">
+        <is>
+          <t>Where an EOW is the cause of a chain reaction (EOW leading to soil washout leading to subsidence), record the claim under the nature of the physical damage (subsidence) not the trigger mechanism; when applying a lower excess as a goodwill gesture (e.g. EOW excess rather than subsidence excess), make explicitly clear in writing that the excess reference does not alter the claim category for recording purposes</t>
+        </is>
+      </c>
+      <c r="T55" s="5" t="inlineStr">
+        <is>
+          <t>IF eow_causes_soil_washout AND soil_washout_causes_building_movement THEN physical_damage_type = subsidence AND claim_category = subsidence; IF settlement_form_references_eow_only_for_excess_purposes THEN eow_reference_does_not_change_claim_recording_category</t>
+        </is>
+      </c>
+      <c r="U55" s="4" t="inlineStr">
+        <is>
+          <t>DRN7112734.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="120" customHeight="1">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>EOW-055</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>DRN7147115</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Legal &amp; General Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>30 Dec 2018</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>Escape of water from dishwasher discovered November 2017; claim made January 2018; insurer declined citing gradually operating cause (alleged continued dishwasher use) and failure to prevent further damage</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>Dishwasher — water leaking onto the dishwasher's electrical wiring, tripping the electricity supply; Mr C isolated the dishwasher after identifying the source</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J56" s="3" t="inlineStr">
+        <is>
+          <t>Legal and General alleged Mr and Mrs C continued to use the dishwasher after discovering the leak, making the cause gradual (November 2017 to January 2018); relied on loss adjustor's observation of dirty dishes in the dishwasher in March 2018 as evidence of continued use; also alleged failure to take reasonable steps to prevent further damage after discovering the problem</t>
+        </is>
+      </c>
+      <c r="K56" s="3" t="inlineStr">
+        <is>
+          <t>L&amp;G relied on loss adjustor's observation of dirty dishes in dishwasher in March 2018 (no photographs taken); also argued nature of damage (kitchen flooring tiles and unit doors) was consistent with prolonged gradual escape; Mr and Mrs C denied dirty dishes in dishwasher; argued water on electrical wiring would make continued use an electrocution risk — a compelling reason to stop immediately; Mr C was a plumber and isolated the dishwasher's plumbing</t>
+        </is>
+      </c>
+      <c r="L56" s="2" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M56" s="3" t="inlineStr">
+        <is>
+          <t>Legal and General Insurance Limited directed to reconsider the claim in line with remaining policy terms; not to decline on gradually operating cause or failure to prevent further damage grounds; no D&amp;I compensation awarded</t>
+        </is>
+      </c>
+      <c r="N56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O56" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P56" s="3" t="inlineStr">
+        <is>
+          <t>The insurer bears the burden of proving a gradually operating cause exclusion applies — it is not on the policyholder to disprove it; where the policyholder has a compelling rational reason for immediately stopping use of an appliance (water on live electrical wiring creates electrocution risk), continued use is implausible; undocumented observations of an inspector are weak evidence against a specific rational explanation for stopping use; the 2-month gap between discovering the leak and making a claim notification is not itself gradual damage</t>
+        </is>
+      </c>
+      <c r="Q56" s="3" t="inlineStr">
+        <is>
+          <t>Photographs of the dirty dishes in the dishwasher at the March 2018 inspection; independent report confirming whether the nature of the damage was consistent with prolonged gradual escape or a shorter period of standing water under flooring</t>
+        </is>
+      </c>
+      <c r="R56" s="3" t="inlineStr">
+        <is>
+          <t>Mr and Mrs C had a compelling rational reason not to continue using the dishwasher — water on electrical wiring creates an electrocution risk; L&amp;G's loss adjustor saw dirty dishes but took no photographs; it is implausible that Mr and Mrs C would knowingly cause continuing water damage and risk electrocution; L&amp;G failed to demonstrate that continued use occurred; the 2-month notification delay did not constitute gradual damage; L&amp;G did not discharge its burden of proving the exclusion applied</t>
+        </is>
+      </c>
+      <c r="S56" s="3" t="inlineStr">
+        <is>
+          <t>When declining on gradually operating cause for an appliance leak, the insurer must produce positive evidence of continued use — circumstantial observations without photographs are insufficient where the policyholder provides a rational explanation for stopping; consider whether the policyholder had a rational safety reason to stop (e.g. electrical hazard) — this substantially undermines the gradual use theory; notification delay alone does not establish gradual damage</t>
+        </is>
+      </c>
+      <c r="T56" s="3" t="inlineStr">
+        <is>
+          <t>IF gradual_cause_exclusion_invoked AND policyholder_had_safety_reason_to_stop AND insurer_evidence_is_undocumented_observation THEN insurer_fails_burden_of_proof; IF notification_delay_2_months AND leak_isolated_at_discovery THEN gradual_cause_exclusion = NOT established</t>
+        </is>
+      </c>
+      <c r="U56" s="2" t="inlineStr">
+        <is>
+          <t>DRN7147115.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="120" customHeight="1">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>EOW-056</t>
+        </is>
+      </c>
+      <c r="B57" s="4" t="inlineStr">
+        <is>
+          <t>DRN7411842</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>Ageas Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D57" s="4" t="inlineStr"/>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>Escape of water at a landlord's rental property between tenancies; insurer declined under unoccupied and untenanted exclusion; owners visited regularly for decoration works but this was not considered occupancy under the landlord's policy definition</t>
+        </is>
+      </c>
+      <c r="F57" s="5" t="inlineStr">
+        <is>
+          <t>Escape of water during the period between tenancies in January 2013 (specific physical source not identified — dispute focuses on the occupancy exclusion)</t>
+        </is>
+      </c>
+      <c r="G57" s="4" t="inlineStr">
+        <is>
+          <t>Residential home (landlord's policy — between tenancies)</t>
+        </is>
+      </c>
+      <c r="H57" s="4" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I57" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J57" s="5" t="inlineStr">
+        <is>
+          <t>Ageas declined under the EOW unoccupied exclusion — property defined as not lived in by a Tenant; no tenant since August 2012; owners' weekend visits for decoration did not constitute occupancy; additionally, policy required heating or drainage in the November to March period if tenants away 14+ days — this condition would also exclude cover</t>
+        </is>
+      </c>
+      <c r="K57" s="5" t="inlineStr">
+        <is>
+          <t>Mr and Mrs K argued their weekend visits (including overnight stays with beds and cooking equipment) constituted occupancy; Ageas countered that a landlord's policy is designed for tenanted properties and owner visits do not satisfy the tenancy-based occupancy definition; FOS confirmed that occupancy on a landlord's policy requires everyday activities on a regular basis such that a property is considered in the ordinary sense to be lived in — decoration visits do not meet this test; additionally, Ageas confirmed it would have restricted cover had it known the property was untenanted</t>
+        </is>
+      </c>
+      <c r="L57" s="4" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M57" s="5" t="inlineStr">
+        <is>
+          <t>FOS did not uphold — the unoccupied exclusion was properly applied; on a landlord's policy, occupancy requires tenancy by a tenant; owner's decoration visits do not constitute occupancy; the heating and drainage condition (separate November to March condition) would also have excluded cover even if visits were treated as occupancy; no award directed</t>
+        </is>
+      </c>
+      <c r="N57" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O57" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P57" s="5" t="inlineStr">
+        <is>
+          <t>On a landlord's insurance policy, occupied means tenanted — the occupancy definition is tailored to the purpose of the policy (cover for a tenanted residential property); owner's periodic visits for decoration works do not constitute occupancy under a landlord's policy; occupancy requires everyday activities on a regular basis as a primary residence; a landlord's policy November to March condition requiring heating and drainage when tenants are away 14+ days is a separate exclusion that may independently apply</t>
+        </is>
+      </c>
+      <c r="Q57" s="5" t="inlineStr">
+        <is>
+          <t>Evidence of whether the November to March heating and drainage condition was met during the period in question; evidence of whether the property had been presented as tenanted or untenanted at the November 2012 renewal</t>
+        </is>
+      </c>
+      <c r="R57" s="5" t="inlineStr">
+        <is>
+          <t>A landlord's policy is designed for tenanted premises — the definition of occupancy as tenancy is not unusual or unreasonable; owner visits for decoration are not everyday residential activities; even if visits counted as occupancy, the November to March heating and drainage condition would independently have excluded cover; Ageas would have restricted cover had it known the property was untenanted — this further supports the decline; broker conduct at point of sale is outside the scope of the insurer's complaint</t>
+        </is>
+      </c>
+      <c r="S57" s="5" t="inlineStr">
+        <is>
+          <t>On landlord's policies, always check whether the property is currently tenanted before accepting an EOW claim — the occupancy definition is tied to tenancy; notify insurers promptly whenever a property becomes untenanted between lettings; check for seasonal heating and drainage conditions that apply between November and March independently of the vacancy exclusion</t>
+        </is>
+      </c>
+      <c r="T57" s="5" t="inlineStr">
+        <is>
+          <t>IF landlords_policy AND property_untenanted_30_days_plus THEN unoccupied_exclusion = applicable_regardless_of_owner_visits; IF november_to_march AND tenants_absent_14_days_plus AND heating_not_maintained THEN seasonal_exclusion = also_applicable</t>
+        </is>
+      </c>
+      <c r="U57" s="4" t="inlineStr">
+        <is>
+          <t>DRN7411842.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="120" customHeight="1">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>EOW-057</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>DRN9891691</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>UK Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>7 Sep 2015</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>Escape of water from bathroom waste pipe; contents claim — electrical items accepted; soft furnishings (sofa, rug, carpet) declined as damage not consistent with EOW; upholsterer's report cost also disputed</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t>Bathroom waste pipe escape of water</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Partial</t>
+        </is>
+      </c>
+      <c r="J58" s="3" t="inlineStr">
+        <is>
+          <t>UKI accepted the claim for electrical items; declined sofa, rug and carpet on the basis that damage was not consistent with EOW — loss assessor found carpet stain was pre-existing (no ceiling staining above it), rug damage (curling, bald patches) was not attributable to EOW, and upholsterer's report for sofa stated EOW causation was only a possibility; damage more consistent with wear and tear and general usage</t>
+        </is>
+      </c>
+      <c r="K58" s="3" t="inlineStr">
+        <is>
+          <t>Loss assessor found no ceiling staining above the carpet stain (indicating pre-existing damage, not EOW); rug showed wear-consistent damage (curling edges, bald patches); upholsterer's report stated the sofa damage was only a possibility from EOW and noted oil and dirt staining; UKI policy required written estimates to be provided at the policyholder's expense; Ms H claimed she was verbally told the items would be covered but no record of this conversation existed on the insurer's file</t>
+        </is>
+      </c>
+      <c r="L58" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M58" s="3" t="inlineStr">
+        <is>
+          <t>FOS did not uphold — damage to soft furnishings was not established as caused by the EOW; absence of ceiling staining above the carpet stain supported pre-existing damage; upholsterer's only a possibility was insufficient; policy required estimates at policyholder's expense; no record of verbal commitment found; no award directed</t>
+        </is>
+      </c>
+      <c r="N58" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O58" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P58" s="3" t="inlineStr">
+        <is>
+          <t>A policyholder bears the burden of demonstrating that each claimed item was damaged by the EOW; absence of ceiling staining above a carpet stain is strong physical evidence that the stain pre-dates the EOW; an expert or specialist report stating EOW causation is only a possibility is insufficient to discharge the policyholder's burden; where a policy requires written estimates to be provided at the policyholder's expense, the insurer is not liable to reimburse the cost of reports or assessments commissioned by the policyholder; a claimed verbal commitment must be evidenced — absence from the insurer's records makes it implausible</t>
+        </is>
+      </c>
+      <c r="Q58" s="3" t="inlineStr">
+        <is>
+          <t>Contemporaneous photographs of carpet, rug and sofa taken immediately after the EOW before cleaning was attempted; evidence that ceiling above the carpet area was affected by the EOW; upholsterer's report stating a definitive rather than qualified opinion on causation</t>
+        </is>
+      </c>
+      <c r="R58" s="3" t="inlineStr">
+        <is>
+          <t>No ceiling staining above the carpet orange stain — physical evidence contradicting EOW causation; rug damage (curling edges, bald patches) consistent with wear and tear rather than water damage; upholsterer's report noted oil and dirt staining and gave only a qualified possibility opinion — insufficient burden discharge; Mr H attempted cleaning before inspection, reducing available physical evidence; no record of verbal commitment on insurer file; the policyholder did not act to her detriment on the alleged verbal commitment</t>
+        </is>
+      </c>
+      <c r="S58" s="3" t="inlineStr">
+        <is>
+          <t>For EOW contents claims, photograph all claimed items before any cleaning or removal — post-EOW cleaning significantly weakens causation evidence; absence of ceiling staining above soft furnishing damage is a key indicator of pre-existing damage; expert or specialist reports must give a definitive opinion to discharge the policyholder's burden — a possibility is insufficient; verbal commitments by insurers cannot be relied upon without documentary evidence</t>
+        </is>
+      </c>
+      <c r="T58" s="3" t="inlineStr">
+        <is>
+          <t>IF carpet_stain_alleged_from_eow AND no_ceiling_staining_above_stain THEN carpet_stain = pre_existing_not_eow; IF expert_report_states_eow_causation_only_a_possibility THEN policyholder_burden = NOT discharged; IF verbal_commitment_claimed AND no_record_on_insurer_file AND no_detrimental_reliance THEN verbal_commitment_claim = fails</t>
+        </is>
+      </c>
+      <c r="U58" s="2" t="inlineStr">
+        <is>
+          <t>DRN9891691.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>